<commit_message>
fase1: pone al día el tracker — S1 (SIS-A-15, SIS-B-03, SIS-F-18, SIS-C-10) y S3 (MAT-D7, SIS-F-03, SIS-F-14, MAT-O20) cerrados
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145f2tyW9URgf61iyJrf1n7
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clusters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan_Fases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflictos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Clusters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Plan_Fases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Conflictos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hallazgos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hallazgos'!$A$1:$L$235</definedName>
@@ -2768,11 +2768,19 @@
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>d33a38a</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2872,11 +2880,19 @@
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr"/>
-      <c r="L19" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>d33a38a</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -9000,11 +9016,19 @@
       </c>
       <c r="J141" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K141" s="6" t="inlineStr"/>
-      <c r="L141" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K141" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L141" s="6" t="inlineStr">
+        <is>
+          <t>d33a38a</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -9204,11 +9228,19 @@
       </c>
       <c r="J145" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K145" s="6" t="inlineStr"/>
-      <c r="L145" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K145" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L145" s="6" t="inlineStr">
+        <is>
+          <t>d33a38a</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -11020,11 +11052,19 @@
       <c r="I183" s="6" t="inlineStr"/>
       <c r="J183" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K183" s="6" t="inlineStr"/>
-      <c r="L183" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K183" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L183" s="6" t="inlineStr">
+        <is>
+          <t>59440a9 + 8b033b6</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="5" t="inlineStr">
@@ -11070,11 +11110,19 @@
       <c r="I184" s="6" t="inlineStr"/>
       <c r="J184" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K184" s="6" t="inlineStr"/>
-      <c r="L184" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K184" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L184" s="6" t="inlineStr">
+        <is>
+          <t>08ba613</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="inlineStr">
@@ -12758,11 +12806,19 @@
       <c r="I218" s="6" t="inlineStr"/>
       <c r="J218" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K218" s="6" t="inlineStr"/>
-      <c r="L218" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K218" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L218" s="6" t="inlineStr">
+        <is>
+          <t>219f584</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="5" t="inlineStr">
@@ -13108,11 +13164,19 @@
       <c r="I225" s="6" t="inlineStr"/>
       <c r="J225" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K225" s="6" t="inlineStr"/>
-      <c r="L225" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K225" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1)</t>
+        </is>
+      </c>
+      <c r="L225" s="6" t="inlineStr">
+        <is>
+          <t>3c526b4</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(housekeeping): marca como N/A las 10 filas sin cluster (9 OK + 1 retirada)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145f2tyW9URgf61iyJrf1n7
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -13218,10 +13218,14 @@
       <c r="I226" s="6" t="inlineStr"/>
       <c r="J226" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K226" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K226" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L226" s="6" t="inlineStr"/>
     </row>
     <row r="227">
@@ -13264,10 +13268,14 @@
       <c r="I227" s="6" t="inlineStr"/>
       <c r="J227" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K227" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K227" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L227" s="6" t="inlineStr"/>
     </row>
     <row r="228">
@@ -13310,10 +13318,14 @@
       <c r="I228" s="6" t="inlineStr"/>
       <c r="J228" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K228" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K228" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L228" s="6" t="inlineStr"/>
     </row>
     <row r="229">
@@ -13356,10 +13368,14 @@
       <c r="I229" s="6" t="inlineStr"/>
       <c r="J229" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K229" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K229" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L229" s="6" t="inlineStr"/>
     </row>
     <row r="230">
@@ -13402,10 +13418,14 @@
       <c r="I230" s="6" t="inlineStr"/>
       <c r="J230" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K230" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K230" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L230" s="6" t="inlineStr"/>
     </row>
     <row r="231">
@@ -13448,10 +13468,14 @@
       <c r="I231" s="6" t="inlineStr"/>
       <c r="J231" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K231" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K231" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L231" s="6" t="inlineStr"/>
     </row>
     <row r="232">
@@ -13494,10 +13518,14 @@
       <c r="I232" s="6" t="inlineStr"/>
       <c r="J232" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K232" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K232" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L232" s="6" t="inlineStr"/>
     </row>
     <row r="233">
@@ -13540,10 +13568,14 @@
       <c r="I233" s="6" t="inlineStr"/>
       <c r="J233" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K233" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K233" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L233" s="6" t="inlineStr"/>
     </row>
     <row r="234">
@@ -13586,10 +13618,14 @@
       <c r="I234" s="6" t="inlineStr"/>
       <c r="J234" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K234" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K234" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L234" s="6" t="inlineStr"/>
     </row>
     <row r="235">
@@ -13632,10 +13668,14 @@
       <c r="I235" s="6" t="inlineStr"/>
       <c r="J235" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K235" s="6" t="inlineStr"/>
+          <t>N/A (sin trabajo)</t>
+        </is>
+      </c>
+      <c r="K235" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría normativa</t>
+        </is>
+      </c>
       <c r="L235" s="6" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fase1(S2): el tracker cita también el commit de cierre de la auditoría adversarial
Los 32 IDs de C08 pasan a citar `3ea627c + 7266bfe`: el trabajo y los tres
restos que la auditoría adversarial encontró después. Sin la segunda
referencia, quien siga el rastro desde la matriz se queda en un árbol donde
la guardia del conteo de Fase 5 todavía tenía el hueco.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014C1uAB8vHEN5cjmjBkLt3M
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -2000,7 +2000,7 @@
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="L46" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="L47" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="L58" s="6" t="inlineStr">
         <is>
-          <t>3ea627c — Docstrings resincronizados (v_max_*, conteo de M2, ejemplo de MD). El VALOR de h_relleno_min_concreto_tmc queda en el paquete del conflicto #5 (C01: MAT-D3/D4, NOR-VAC-01): aqui solo se describe su estado, no se cierra el vacio.</t>
+          <t>3ea627c + 7266bfe — Docstrings resincronizados (v_max_*, conteo de M2, ejemplo de MD). El VALOR de h_relleno_min_concreto_tmc queda en el paquete del conflicto #5 (C01: MAT-D3/D4, NOR-VAC-01): aqui solo se describe su estado, no se cierra el vacio.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="L65" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="L69" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="L98" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7132,7 +7132,7 @@
       </c>
       <c r="L102" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="L104" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7352,7 +7352,7 @@
       </c>
       <c r="L106" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7410,7 @@
       </c>
       <c r="L107" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7468,7 +7468,7 @@
       </c>
       <c r="L108" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
       </c>
       <c r="L109" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="L113" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="L116" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="L119" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10538,7 @@
       </c>
       <c r="L169" s="6" t="inlineStr">
         <is>
-          <t>3ea627c — Ficha de cobertura (CONFIRMA). Reverificado sobre las dos memorias generadas tras el cambio: sin citas truncadas, plantillas sin numerales, analogia [N-&gt;] declarada, adopcion de Clase F impresa, avisos de trazabilidad y "(proyecto no declarado)".</t>
+          <t>3ea627c + 7266bfe — Ficha de cobertura (CONFIRMA). Reverificado sobre las dos memorias generadas tras el cambio: sin citas truncadas, plantillas sin numerales, analogia [N-&gt;] declarada, adopcion de Clase F impresa, avisos de trazabilidad y "(proyecto no declarado)".</t>
         </is>
       </c>
     </row>
@@ -10880,7 +10880,7 @@
       </c>
       <c r="L176" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -11454,7 +11454,7 @@
       </c>
       <c r="L187" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -11512,7 +11512,7 @@
       </c>
       <c r="L188" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -11620,7 +11620,7 @@
       </c>
       <c r="L190" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12266,7 +12266,7 @@
       </c>
       <c r="L203" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12574,7 +12574,7 @@
       </c>
       <c r="L209" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12632,7 +12632,7 @@
       </c>
       <c r="L210" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12740,7 +12740,7 @@
       </c>
       <c r="L212" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12798,7 +12798,7 @@
       </c>
       <c r="L213" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="L214" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>
@@ -13172,7 +13172,7 @@
       </c>
       <c r="L220" s="6" t="inlineStr">
         <is>
-          <t>3ea627c</t>
+          <t>3ea627c + 7266bfe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S4): el tracker cita también el commit de cierre de la auditoría adversarial
NOR-VAC-01 lleva además la nota CONTRA LA FICHA: su propia transcripción del
segundo término de la Tabla 12.6.6.3-1 («√Bc/8») es errónea — la tabla dice
`B′c/8`, y `B′c` es la *out-to-out vertical rise of pipe*, que en conducto
circular es `Bc`. Quien lea la ficha sin abrir el PDF repite el error, que es
exactamente lo que pasó aquí.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeazcCh1jvGdbb8R8QC9Q9
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -2058,7 +2058,7 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>3d59da0 — verificado leyendo el PDF: ASTM A760/A760M-10, Tabla 1 'Tamaños de tuberia', pag. 3, tabula de 100 a 3600 mm; 2100 mm es una fila mas. El tope se reetiqueta como de catalogo ('D_max_catalogo' [A]) y V9 y el motivo de descarte de MD lo dicen asi.</t>
+          <t>3d59da0 — verificado leyendo el PDF: ASTM A760/A760M-10, Tabla 1 'Tamaños de tuberia', pag. 3, tabula de 100 a 3600 mm; 2100 mm es una fila mas. El tope se reetiqueta como de catalogo ('D_max_catalogo' [A]) y V9 y el motivo de descarte de MD lo dicen asi. || dbaa501 — A760 Tabla 1 arranca en 100 mm (4 in), no en 150; corregido en 'diametros_normalizados'.</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>3d59da0 — el vacio no era un vacio. Se transcribe la Tabla 12.6.6.3-1 de AASHTO LRFD (Art. 12.6.6.3, pag. 12-22) en el criterio 'cobertura_minima_aashto' [C] y h_rec pasa a calcularse como el mayor entre el minimo de EG-2013 (solo HDPE) y esa cobertura. Se RETIRA 'h_relleno_min_concreto_tmc'. Que fila aplica lo decide 'condicion_pavimento' [A], sin valor, que bloquea; el Bc del concreto necesita 'espesor_pared_conducto' [A], sin valor, que tambien bloquea.</t>
+          <t>3d59da0 — el vacio no era un vacio. Se transcribe la Tabla 12.6.6.3-1 de AASHTO LRFD (Art. 12.6.6.3, pag. 12-22) en el criterio 'cobertura_minima_aashto' [C] y h_rec pasa a calcularse como el mayor entre el minimo de EG-2013 (solo HDPE) y esa cobertura. Se RETIRA 'h_relleno_min_concreto_tmc'. Que fila aplica lo decide 'condicion_pavimento' [A], sin valor, que bloquea; el Bc del concreto necesita 'espesor_pared_conducto' [A], sin valor, que tambien bloquea. || dbaa501 — la transcripcion de la Tabla 12.6.6.3-1 se rehizo sobre la celda RENDERIZADA tras la auditoria adversarial: la fila del concreto dice "Bc/8 or B'c/8, whichever is greater, &gt;= 12.0 in.", no "sqrt(Bc)/8" como transcribe la propia ficha NOR-VAC-01 (la prima de B'c es un glifo de SymbolMT que la extraccion de texto rompe). B'c es la "out-to-out vertical rise of pipe", que en conducto circular es Bc, de modo que el maximo se reduce a Bc/8. Cae con la lectura falsa la rama sqrt y el factor pie-metro que se habian introducido. NOTA CONTRA LA FICHA: su transcripcion del segundo termino es erronea.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S5): pone al día el tracker — los 13 hallazgos de C05
Estado / Responsable / Commit de MAT-D1, MAT-O13, MAT-O14, SIS-A-06,
NOR-HID-03, NOR-HID-04, NOR-HID-06, NOR-HID-07, NOR-HID-08, NOR-HID-10,
NOR-HID-11, NOR-HID-12 y NOR-MEM-01. Cada fila cita el commit de cierre y, en
las seis que la auditoría adversarial tocó, también el de la corrección.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsvPPjkZewHY7FK8m25JaS
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -2272,11 +2272,19 @@
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — V2 deja de leer la rama n_min. `modelos.TiranteNormal` y `modelos.ResultadoHidraulico` retiran el campo `V` y llevan dos: `V_erosion` (n_min, estimacion ALTA) y `V_sedimentacion` (n_max, estimacion BAJA), las dos sobre la MISMA geometria de Brent. `M5.v2_velocidad_minima` consume `V_sedimentacion`; `v3_velocidad_maxima` y Laushey (cli._fase_6 -&gt; M6) consumen `V_erosion`. No hay campo neutro que permita elegir mal en silencio. Recomputado a mano: D=0.90, y/D=0.75 (theta=4pi/3), S=5e-5, concreto -&gt; A=0.511800 m2, R=0.271518 m, V(n_max)=0.228073 m/s y V(n_min)=0.296495 m/s con Q=0.116728 m3/s: V2 pasa de 'cumple' a 'NO cumple', que es lo correcto. `Material.n_para_velocidad` se renombra `n_para_velocidad_maxima` (los terminos de la Sec. 4.1 de la hoja de ruta) y se agrega `n_para_velocidad_minima`.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -4136,11 +4144,19 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — `DIAMETRO_MIN` lleva ahora el texto literal del num. 4.1.1.3.4 a) (`DIAMETRO_MIN_TEXTO`, pag. impresa 72) y su ambito (`DIAMETRO_MIN_AMBITO`), con las dos condiciones: 'carreteras de alto volumen de transito' -- que el proyecto NO puede afirmar porque la clase de via no esta cerrada, y aplicar el piso igual queda declarado como adopcion conservadora -- y 'salvo en cruces de canales de riego', que es la Familia C de este expediente. El codigo ya no le aplicaba el piso a la Familia C (`M2.materiales_candidatos` devuelve tupla vacia), pero la razon escrita era solo la forma de la seccion; ahora la excepcion normativa esta en el docstring del modulo, en la funcion y en la `fuente` de 'diametros_normalizados'. Se cierra el defecto de CITA; el piso nunca llegaba a la Familia C por la via de calculo. || 76791d0 -- la auditoria adversarial mostro que estaba cerrado solo en `DIAMETRO_MIN`, que no tiene consumidor: la cadena viva conservaba la formula que la ficha cita como defecto. Corregidos `D_INICIO` ('minimo normativo MTC' a secas), el docstring 'Sec. 3.2 - Catalogo de diametros' de M2 y la fila del manifiesto. Y se retira una afirmacion FALSA que este mismo cluster habia introducido en DIAMETRO_MIN_AMBITO -- que aplicar el piso 'exige mas seccion, nunca menos' y por eso es conservador --: con concreto, S=0.001 y Q=0.0035 m3/s, D=0.75 cumple V2 con 0.2554 m/s y D=0.90 NO cumple con 0.2488. Mas diametro favorece a V1 y perjudica a V2.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -4182,11 +4198,19 @@
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — La frase 'el rango recorre la calidad del revestimiento' sale de la cita y pasa a declararse como INTERPRETACION DEL PROYECTISTA en `constantes_normativas.TABLA_10_INTERPRETACION_PROYECTO`, que M11 imprime separada, en su propio aviso. La `fuente` de 'v_max_concreto_eleccion', `M5.NUMERAL_V3` y la nota de la §1 del manifiesto separan ahora lo que la fuente sostiene (los dos numeros son maximos: lo dice el titulo y el rotulo 'VELOCIDAD (M/S)') de lo que pone el proyecto, y citan los dos hechos que juegan en contra de la lectura de acabados: la frase que introduce la tabla ('un rango, cuyos limites se describen a continuacion') y la fila de mamposteria con un solo valor.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -4448,11 +4472,19 @@
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K49" s="6" t="inlineStr"/>
-      <c r="L49" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — Cerrado sobre el PRODUCTO, que era donde fallaba. El matiz viajaba solo dentro de `M5.NUMERAL_V2`, o sea dentro de la tabla de verificaciones del punto, que no se imprime si el punto no llego a evaluarse -- y no llega, porque 'homogeneidad_serie_fen' bloquea el Q de la Familia A. Se agrega `constantes_normativas.UMBRALES_DE_VERIFICACION` (V1, V2, V3, TR y D_min con numeral, caracter, texto literal y lo que el proyecto hace con cada uno), `M11.bloque_umbrales()` y el marcador %%bloque_umbrales en las dos plantillas, en la seccion nueva '0-ter. Umbrales normativos y su caracter', que se imprime siempre. Medido sobre la memoria generada con tests/ejemplo_puntos.csv en los dos alcances: 'recomend' pasa de 0 a 7 apariciones y 'sedimentaci' de 0 a 3. || 76791d0 -- ademas, la memoria imprimia 'num. MC-HHD (...), num. 3.6' porque M11 anteponia 'num.' a un NUMERAL_TR que ya lo trae; y NUMERAL_V3 remitia a un simbolo de codigo que un revisor con el PDF no puede resolver.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -5318,11 +5350,19 @@
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K66" s="6" t="inlineStr"/>
-      <c r="L66" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K66" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L66" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — La Tabla N 02 se transcribe COMPLETA (seis filas) con su titulo literal 'VALORES MAXIMOS RECOMENDADOS de riesgo admisible de obras de drenaje', el texto que la introduce ('se recomienda utilizar como maximo') y las dos notas al pie, incluida la que asigna la decision al Propietario. El caracter viaja al punto de uso: `M1.NUMERAL_TR` y el `fundamento` de `PeriodoRetorno` declaran que son maximos recomendados adoptados por el proyecto y que adoptarlos es -- al reves que en V1 y V2 -- el extremo MENOS conservador del margen concedido. NO se reetiqueta [N]-&gt;[A]: por la regla de CLAUDE.md la TABLA es [N] y lo que es [A] es la eleccion, que para la Familia A ya vive en 'umbral_area_quebrada_importante_ha' (sin valor, bloquea) y para la Familia B la fija la Sec. 2.3. Lo que faltaba era el caracter declarado, y es lo que se cierra. || 76791d0 -- cerrado en parte hasta la auditoria adversarial: `NUMERAL_TR` imprimia 'mientras el Propietario no declare otros' y no habia via para declararlos. Entra 'riesgo_admisible_propietario' [A] opcional (no bloquea; sin declarar rigen los maximos de la tabla), leido por `M1._riesgo_del_propietario`, que solo admite ENDURECER el techo: R por encima del maximo recomendado o n por debajo del de la nota al pie es DatoInvalidoError. Verificado: R=0.20 con n=25 lleva el TR de 71 a 113 anios.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -5368,11 +5408,19 @@
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K67" s="6" t="inlineStr"/>
-      <c r="L67" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K67" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L67" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — Mismo cierre que MAT-O13: V1 y V2 salen del mismo tipo de frase ('se recomienda') y ahora los dos numerales lo dicen. Ademas el caracter de los dos viaja a la memoria por una via que no depende de que el punto se evalue (`UMBRALES_DE_VERIFICACION`).</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -5414,11 +5462,19 @@
       <c r="I68" s="6" t="inlineStr"/>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K68" s="6" t="inlineStr"/>
-      <c r="L68" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L68" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — `TABLA_09_FILAS` transcribe las TRES columnas (MINIMO / NORMAL / MAXIMO) y las DOS subfilas de metal corrugado con su nombre literal; `MANNING` pasa a ser vista derivada (n_min, n_max), no una copia. Las claves declaran la subfila: 'metal_corrugado_dren_aguas_lluvias' y 'metal_corrugado_subdren', 'concreto_tubo_recto', 'madera_duelas'. `M2._MANNING_CLAVE` declara que material toma que subfila y por que (una alcantarilla es dren de aguas lluvias, no sub-dren; el concreto es tubo recto y libre de basuras, no tubo de alcantarillado con camaras). Por que el calculo no usa la columna NORMAL queda escrito: la regla de doble n pide los dos extremos, no el valor corriente. `Material.fila_manning` lleva la fila literal a la memoria.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -6070,11 +6126,19 @@
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K80" s="6" t="inlineStr"/>
-      <c r="L80" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L80" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — `M5.NUMERAL_V1` deja de ser el numeral pelado: lleva RD, pag. impresa 79, el texto literal del 4.1.1.3.7 b) y el matiz de RECOMENDACION, igual que NUMERAL_V2, mas la declaracion de que el proyecto lo aplica como umbral duro. El comportamiento no cambia. Verificado contra el PDF: 'Se recomienda que el diseño hidraulico considere como minimo el 25 % de la altura, diametro o flecha de la estructura' (pag. impresa 79).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -6124,11 +6188,19 @@
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K81" s="6" t="inlineStr"/>
-      <c r="L81" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L81" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — 'v_max_tmc' y 'v_max_hdpe' pasan de 4.6 a 4.572 m/s: 15 ft x 0.3048 = 4.572 exactos, y 4.6 quedaba 0.6 % POR ENCIMA de un techo que el propio criterio declara duro. Los dos criterios declaran ademas que la Tabla 8-4 de WSDOT NO esta en normas/ y que la cita no es auditable contra el repositorio. DEFECTO REPORTADO CONTRA LA HOJA DE RUTA, no corregido aqui: la fila V3 de la tabla de la Fase 5 de docs/hoja_de_ruta_alcantarillas_v8.md sigue diciendo 'TMC y HDPE: PPI/FHWA, valor por extraer' -- el criterio esta cerrado y la fuente que lo cerro es WSDOT, no PPI/FHWA. || 76791d0 -- tres referencias cruzadas se quedaron en 4.6 (el modo de fallo de SIS-A-20): docstring de M2, `verificacion_pendiente` de 'clases_producto_por_relleno' y un docstring de test.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -10486,11 +10558,19 @@
       <c r="I166" s="6" t="inlineStr"/>
       <c r="J166" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K166" s="6" t="inlineStr"/>
-      <c r="L166" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K166" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L166" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — El titulo de la Tabla N 10 se transcribe con la unidad -- 'Velocidades maximas admisibles (m/s) en conductos revestidos' -- en los tres sitios que lo citaban sin ella: `constantes_normativas.TABLA_10_TITULO`, `M5.NUMERAL_V3` y la `fuente` de 'v_max_concreto_eleccion'. Verificado contra el PDF, pag. impresa 76. || 76791d0 -- `bloque_umbrales` reintrodujo el mismo defecto que cerraba: rotulaba 'Texto literal' dos composiciones que no lo eran (prosa del proyecto en TR, la tabla reformateada en V3) y el titulo de la Tabla N 02 no iba verbatim. `texto` pasa a ser tupla de citas verbatim impresas por separado; lo que no es cita va en `transcripcion`.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
@@ -10532,11 +10612,19 @@
       <c r="I167" s="6" t="inlineStr"/>
       <c r="J167" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K167" s="6" t="inlineStr"/>
-      <c r="L167" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K167" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L167" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — Los nombres de fila se transcriben completos y literales. Tabla N 02 (`TABLA_02_FILAS`): 'Alcantarillas de paso de quebradas importantes y badenes' y 'Alcantarillas de paso quebradas menores y descarga de agua de cunetas', ademas de las otras cuatro filas de la tabla. Tabla N 10 (`TABLA_10_FILAS`): 'Mamposteria de piedra y concreto', y su valor deja de escribirse (2.0, 2.0) -- un par que la fuente no imprime -- para quedar en (2.0,). `M5.v3_velocidad_maxima` toma `max()` de la fila en vez de desempaquetar dos valores. || 76791d0 -- la transcripcion se anunciaba completa y dejaba la fila 'Puentes (*)' con su marcador y sin la nota. Se agregan TABLA_02_NOTA_PUENTES y TABLA_02_NOTA_IMPORTANCIA, y TABLA_02_NOTAS reune las cuatro.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="inlineStr">
@@ -10916,11 +11004,19 @@
       <c r="I175" s="6" t="inlineStr"/>
       <c r="J175" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K175" s="6" t="inlineStr"/>
-      <c r="L175" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K175" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L175" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — `Material.v_max_rango: Optional[Tuple[float,float]]` se parte en dos campos que no se confunden: `v_max_tabla10: Optional[Tuple[float, ...]]` (la fila literal de la Tabla N 10; None si el material no tiene fila) y `v_max_adoptado: Optional[float]` (el techo escalar del criterio [C] de TMC y HDPE). Ya no hay un campo anotado como par que transporte un escalar. El docstring de `v_max_definida` deja de decir 'False para TMC y HDPE' -- hoy devuelve True para los tres -- y explica cuando vuelve a False.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="5" t="inlineStr">
@@ -12106,11 +12202,19 @@
       <c r="I198" s="6" t="inlineStr"/>
       <c r="J198" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K198" s="6" t="inlineStr"/>
-      <c r="L198" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K198" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S5)</t>
+        </is>
+      </c>
+      <c r="L198" s="6" t="inlineStr">
+        <is>
+          <t>00da460 — `DIAMETRO_MIN_SELVA_ALTA` se renombra `DIAMETRO_MIN_TMC_SELVA_ALTA_RECOMENDADO` -- dos de las tres restricciones en el nombre -- y se acompaña del texto literal (`..._TEXTO`: 'Se recomienda utilizar... como diametro minimo alcantarillas TMC Ø 48"') y de las cuatro caracteristicas geomorfologicas que el numeral exige (`..._CONDICIONES`), verificadas sobre el PDF, pag. impresa 79. Sigue sin consumidor de calculo y sigue declarado en CONSTANTES_DE_REFERENCIA.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S7): pone al dia el tracker — los 4 hallazgos de C13
MAT-D9, MAT-O5, MAT-O6 y SIS-A-21 pasan a Cerrado en la hoja `Hallazgos` de
docs/auditorias/matriz_cruzada_auditorias.xlsx, con responsable y commits, y
cada uno con la evidencia de por que se da por cerrado: el caso numerico
recomputado en MAT-D9, la cita del PDF primario en MAT-O5, el algebra en
MAT-O6 y el consumidor que quedaba sin guarda en SIS-A-21.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019mDzMRmqsZWcD6pvJRAAGR
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -3084,11 +3084,19 @@
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S7)</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>0f3cf28 + 0f63edd — la pendiente deja de elegirse dos veces. `modelos.ResultadoHidraulico` gana el campo obligatorio `S` -- la pendiente CON QUE corrio el diseño --, que `M4.resolver_control` llena con la que recibio, y `M7.compatibilidad_geometrica` PIERDE su parametro `S`: la lee de `resultado.S`. `cli._fase_7` ya no puede omitirla ni discrepar. Caso recomputado a mano: punto con cota de entrada 42.10 msnm, L = 20.0 m, cota de fondo del receptor 41.30 y S_cauce 0.006; con S_conducto declarada 0.045 la caida es 0.900 m, la cota de salida 41.200 y G2 INCUMPLE. Antes esa misma corrida daba caida 0.120 y salida 41.980 con G2 cumplida, o sea el conducto entregando 0.10 m BAJO el fondo del receptor sin que nada lo dijera. La MEMORIA lo imprime ahora, que es donde el hallazgo hacia dano: `M11_reporte._tabla_diseno` saca S en la fila de Hidraulica, al lado de Q, y la CLI en el bloque de Fase 4 (texto y JSON). Antes la unica pendiente del entregable era la columna S_cauce de los datos de partida, que en ese punto NO es la del diseño: la memoria traia 'Pendiente del cauce 0.010 m/m' junto a 'caida 0.900 m' y la caida no se podia recomputar. Verificado sobre la memoria generada.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -5708,11 +5716,19 @@
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K71" s="6" t="inlineStr"/>
-      <c r="L71" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K71" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S7)</t>
+        </is>
+      </c>
+      <c r="L71" s="6" t="inlineStr">
+        <is>
+          <t>0f3cf28 + 0f63edd — defecto documental de la hoja de ruta v8, corregido en la hoja. La fila V4 de la tabla de Fase 5 pasa de «HW &lt;= cota de subrasante - resguardo(CBR)» a «cota de entrada + HW &lt;= cota de subrasante - resguardo(CBR)», con una NOTA DE DATUM en la Sec. 5.1. El codigo nunca lo escribio mal (`M5.v4_carga_entrada` suma `cota_entrada_supuesta`) y ahora su docstring lo dice con el sumando explicito. La forma nivel-contra-nivel se verifico contra el PDF primario (Manual de Suelos, num. 4.5.4, pag. impresa 42): «El nivel superior de la sub rasante debe quedar encima del nivel de la napa freatica como minimo a 0.60 m ...». Los dos terminos que el numeral compara son del mismo tipo.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -5762,11 +5778,19 @@
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K72" s="6" t="inlineStr"/>
-      <c r="L72" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S7)</t>
+        </is>
+      </c>
+      <c r="L72" s="6" t="inlineStr">
+        <is>
+          <t>0f3cf28 + 0f63edd — misma correccion documental en la Sec. 7.A: la segunda condicion del max{} pasa de «HW + resguardo + e_paq» a «cota entrada + HW + resguardo + e_paq», con la equivalencia con V4 escrita en la propia hoja. El algebra se verifico: con e_paq = cota rasante - cota subrasante, «cota rasante &gt;= cota entrada + HW + resguardo + e_paq» es exactamente «cota entrada + HW &lt;= cota subrasante - resguardo». `M7.tamizado_rasante` ya calculaba `por_resguardo = entrada + HW + resguardo + e_paq`. Las cuatro copias de la formula incoherente en docstrings del codigo (`M7` cabecera y `tamizado_rasante`, `modelos.CondicionRasante` y `modelos.TamizadoRasante`) tambien se corrigieron.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -12634,11 +12658,19 @@
       <c r="I204" s="6" t="inlineStr"/>
       <c r="J204" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K204" s="6" t="inlineStr"/>
-      <c r="L204" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K204" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S7)</t>
+        </is>
+      </c>
+      <c r="L204" s="6" t="inlineStr">
+        <is>
+          <t>0f3cf28 + 0f63edd — la resta se escribe una sola vez, con su guarda. Nueva funcion publica `M5_verificaciones.altura_relleno_sobre_clave(punto, material, D)`, que calcula subrasante menos clave fisica y lanza `DatoInvalidoError` sobre 'cota_subrasante' cuando la clave queda al nivel de la subrasante o por encima. La usan `v7_flotacion` y `cli._fase_8`, que antes repetia la resta sin guarda. El hallazgo decia «hoy sin efecto porque M8 se detiene antes», y esa es la razon de cerrarlo ahora: el dia en que 'clases_producto_por_relleno' se declare, la Fase 8 entraria a la tabla de la norma de producto con una altura negativa.</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S9): pone al dia el tracker — los 26 hallazgos de C04
23 Cerrado y 3 Cerrado parcial. Los tres parciales lo son por el conflicto #8,
que es vinculante y prohibe cablear 'clase_sitio' antes de resolver la
premisa: SIS-B-01 cierra la mitad declarativa y no el cableado, SIS-D-01
cierra la incoherencia entre 'F_pga' y 'clase_sitio' y no el cableado, y
NOR-AAS-02 deja la premisa declarada y detenida, que es lo que el conflicto
ordena. Los tres quedan asignados a S13/S14.

Ningun hallazgo de otro cluster se cerro de paso.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KMYF6RZTZKQDrkATvVkHJ1
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -2748,11 +2748,19 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr"/>
-      <c r="L15" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - CIERRA LA MITAD DECLARATIVA, NO EL CABLEADO, y no puede cerrarlo: el conflicto #8 de la seccion 6 del plan es vinculante y prohibe cablear 'clase_sitio' antes de resolver la premisa (S13). Lo que se hizo: dejar escrito en el propio criterio que ningun modulo de produccion lo invoca, que por eso no entra en criterios_usados() ni la memoria imprime la adopcion, y por que cablearlo hoy seria peor -- la memoria declararia formalmente una clasificacion que la fuente no sostiene. QUEDA ABIERTO el cableado, asignado a S14.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2802,11 +2810,19 @@
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr"/>
-      <c r="L16" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - CIERRA LA INCOHERENCIA, NO EL CABLEADO. La tabla ya tiene fila F (con su asterisco y su Nota 2) y 'F_pga' declara sobre que filas se lee y por que la F no esta entre ellas, de modo que las dos defensas dejan de contradecirse. Sigue siendo cierto que solo 'F_pga' llega a la memoria: eso es el cableado de SIS-B-01, prohibido por el conflicto #8 hasta S13/S14.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3578,11 +3594,19 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr"/>
-      <c r="L30" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - LA PREMISA QUEDA DECLARADA Y DETENIDA, que es lo que el conflicto #8 ordena, no resuelta. La justificacion de 'clase_sitio' deja de afirmar que el sitio es Clase F como cosa cerrada y registra lo verificado: el salto 'licuable -&gt; Clase F' no lo escribe ninguno de los dos documentos que el criterio invoca (AASHTO trata la licuefaccion en su Art. 10.5.4.2, por via distinta de la clase de sitio) y quien clasifica los licuables aparte es E.030 en su S5. La discrepancia entre los dos esquemas queda transcrita en `E030_S5_VS_CLASE_F`. RESOLVERLA es S13.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -4622,11 +4646,19 @@
       <c r="I50" s="6" t="inlineStr"/>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr"/>
-      <c r="L50" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La justificacion de 'F_pga' se reescribe: dice de que filas sale la envolvente, y dice por que no estan las otras tres -- A y B son roca, F no da factor sino la exigencia de estudio de la Nota 2 -- cruzando por fin las dos afirmaciones que convivian sin tocarse.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -4726,11 +4758,19 @@
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr"/>
-      <c r="L52" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L52" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - `FACTOR_MURO_TABLA` retirada. El numeral no presenta ninguna tabla y fija un solo valor, permisivo: queda `REDUCCION_KH_POR_DESPLAZAMIENTO = 0.5` y el 1.0 como ausencia de reduccion. El criterio declara si se aplica, no que fila se elige. Corregido tambien el rango '25-50 mm', que redondeaba '1.0 a 2.0 in' y perdia el 'o mas'. Numeral corregido a 2.8.1.1.14.2.2.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -4776,11 +4816,19 @@
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr"/>
-      <c r="L53" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L53" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La afirmacion falsa ('practica corriente; no fijado por el Manual de Puentes') se retira y se sustituye por el texto literal del numeral. Misma correccion que MAT-O11.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -4822,11 +4870,19 @@
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr"/>
-      <c r="L54" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L54" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La afirmacion negativa se retira. La fila F esta transcrita con su asterisco en las cinco columnas y la Nota 2 literal; elegirla es `DatoInvalidoError`, porque no hay numero que leer ahi. La etiqueta [C] que la sostenia se corrige en el criterio: no habia vacio que cubrir.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -5184,11 +5240,19 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K61" s="6" t="inlineStr"/>
-      <c r="L61" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K61" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L61" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Misma correccion que MAT-O2. Se declara por que gana AASHTO y no por preferencia de fuente: con el signo menos K_AE diverge y el caso limite deja de dar el Ka de Coulomb.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -5694,11 +5758,19 @@
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K70" s="6" t="inlineStr"/>
-      <c r="L70" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K70" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L70" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La errata se declara en el punto de uso (`k_ae_mononobe_okabe`), como dato (`K_AE_ERRATA_MANUAL`, con las dos citas y sus paginas) y en la memoria (`condicion_normativa_cabezal`). El codigo NO se toca: sigue a AASHTO, que es lo correcto. Reportado ademas contra la hoja de ruta, que no advertia de la discrepancia.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -6162,11 +6234,19 @@
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K78" s="6" t="inlineStr"/>
-      <c r="L78" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L78" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - El 0.0 pasa a constantes_normativas como `K_V_PRESCRITO` [N], con el texto literal del num. 2.8.1.1.14.2.1 y sus dos casos reservados. El criterio 'k_v' deja de guardar el numero y declara cual de los dos regimenes rige; si rigiera el reservado admite un numero del proyectista, porque el Manual no escribe ninguno para ese caso.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -6518,11 +6598,19 @@
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K84" s="6" t="inlineStr"/>
-      <c r="L84" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L84" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - P_IR = k_h*(W_w + W_s) implementado (`fuerza_inercia_muro`), con W_s definido como lo define la fuente -- suelo inmediatamente encima del muro, incluido el talon -- y no como el relleno del trasdos. La combinacion 100/50 - 50/100 en `demanda_sismica_cabezal`, con el piso 'no menor que el empuje activo estatico' aplicado al segundo caso y el mas desfavorable como gobernante. El ensamble automatico sigue detenido en 'predimensionamiento_cabezal', que es vacio ya declarado y al que se le suma el ancho del talon.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -6614,11 +6702,19 @@
       <c r="I86" s="6" t="inlineStr"/>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K86" s="6" t="inlineStr"/>
-      <c r="L86" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L86" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La fila S5 deja de ser 'referencia muerta': su prohibicion condicionada se transcribe literal (`E030_S5_TEXTO`), se lee con precision -- prohibicion CON salvedad de estudio especifico, ni bloqueo duro ni referencia muerta -- y llega a la memoria por `condicion_normativa_cabezal`.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -6860,11 +6956,19 @@
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K91" s="6" t="inlineStr"/>
-      <c r="L91" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L91" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Misma correccion que MAT-O3: se toma la via 'declarar la hipotesis' de la resolucion, con la desviacion acotada y dicha.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -6914,11 +7018,19 @@
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K92" s="6" t="inlineStr"/>
-      <c r="L92" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L92" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Las dos mitades cerradas: k_h0 deja de ser incondicional (ver MAT-O4) y k_v pasa de [A] a [N] condicionado (ver MAT-O11).</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -7026,11 +7138,19 @@
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K94" s="6" t="inlineStr"/>
-      <c r="L94" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K94" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L94" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Misma correccion que MAT-D6: la seccion que la hoja de ruta citaba para k_h0 exigia el termino omitido, y ahora esta. La hoja de ruta v8 se corrige en su Sec. 9.2, que es donde estaba el defecto.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
@@ -7288,11 +7408,19 @@
       <c r="I99" s="6" t="inlineStr"/>
       <c r="J99" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K99" s="6" t="inlineStr"/>
-      <c r="L99" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K99" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L99" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - El rotulo de la columna se transcribe como lo imprime la tabla, 'PGA &gt; 0.50', y la lectura del borde se declara en el criterio nuevo 'F_pga_lectura_columna_extrema' con su consecuencia dicha: leyendo la columna anterior la fila D daria 1.1 y la envolvente subiria un 10 %. La Nota 1 se implementa (`factor_sitio_desde_tabla` interpola).</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -7338,11 +7466,19 @@
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr"/>
-      <c r="L100" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La regla ni se implementaba ni se descartaba; ahora se implementa Y se descarta con motivo. Ver MAT-O4.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
@@ -7620,11 +7756,19 @@
       <c r="I105" s="6" t="inlineStr"/>
       <c r="J105" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K105" s="6" t="inlineStr"/>
-      <c r="L105" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K105" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L105" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La sensibilidad (0.0, 0.5) se retira, con la razon escrita: sugeria una libertad que el numeral no concede -- el cero es prescrito -- y su comentario ('0.5*k_h') no coincidia ni con su propio extremo ni con lo que prescribe la hoja de ruta.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -7906,11 +8050,19 @@
       </c>
       <c r="J110" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K110" s="6" t="inlineStr"/>
-      <c r="L110" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L110" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Hipotesis declarada como dato (`HIPOTESIS_EMPUJE_BAJO_NF`), con la cita literal de AASHTO 3.11.3 'Presence of Water' (pag. impresa 3-118) y la desviacion cuantificada (+25 % local). Llega a la memoria. No se corrige el calculo: hacerlo exige un peso especifico sumergido que el expediente no tiene, y aplicarlo con el unico gamma declarado ALIVIARIA el empuje sin dato que lo sostenga.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -7960,11 +8112,19 @@
       </c>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K111" s="6" t="inlineStr"/>
-      <c r="L111" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L111" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La clausula ya es representable: `F_PGA_TABLA` transcrita completa incluye las filas A y B, y `coeficiente_sismico_base` tiene las dos ramas. `cimentacion_en_roca()` resuelve cual aplica con las filas que declara 'F_pga', de modo que la rama de roca queda DESCARTADA de forma trazable y se activaria sola si alguien declarase A o B. Destapado ademas que el parentesis del Manual ('1.2 kh0=FpgaPGA') es una segunda errata: gana la prosa.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -8126,11 +8286,19 @@
       <c r="I114" s="6" t="inlineStr"/>
       <c r="J114" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K114" s="6" t="inlineStr"/>
-      <c r="L114" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K114" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L114" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Procedimiento implementado entero: `excentricidad_resultante`, `presion_contacto_base` (Navier dentro del nucleo, distribucion parcial fuera, continuas en e = B/6) y `verificar_excentricidad_sismica`, codigo E6. Y el limite no es el tercio central a secas: depende de gamma_EQ (B/6 a 0.4*B, interpolado), que pasa a ser criterio propio con valor None -- antes vivia como prosa dentro de otro criterio y no podia detener nada.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
@@ -8176,11 +8344,19 @@
       <c r="I115" s="6" t="inlineStr"/>
       <c r="J115" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K115" s="6" t="inlineStr"/>
-      <c r="L115" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K115" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L115" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - La razon se escribe UNA vez, en `M9.FUNCIONES_SIN_CONSUMIDOR`, y la CLI la lee de alli en vez de repetirla en su nota. Mismo patron que `criterios_sin_consumidor`.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -8284,11 +8460,19 @@
       <c r="I117" s="6" t="inlineStr"/>
       <c r="J117" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K117" s="6" t="inlineStr"/>
-      <c r="L117" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K117" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L117" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Misma correccion que SIS-B-17: las siete funciones de armado entran en `FUNCIONES_SIN_CONSUMIDOR` con su insumo bloqueado nombrado.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -8334,11 +8518,19 @@
       <c r="I118" s="6" t="inlineStr"/>
       <c r="J118" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K118" s="6" t="inlineStr"/>
-      <c r="L118" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K118" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L118" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - Misma correccion que SIS-B-17.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
@@ -10266,11 +10458,19 @@
       <c r="I156" s="6" t="inlineStr"/>
       <c r="J156" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K156" s="6" t="inlineStr"/>
-      <c r="L156" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K156" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L156" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - El concepto de `Z_E030` deja de atribuir al Art. 11.1 una cifra que ese articulo no imprime: se transcribe la probabilidad que si escribe y el Tr = 475 se declara como derivacion, con la unica pagina de E.030 donde la cifra aparece literal (Anexo III).</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
@@ -10312,11 +10512,19 @@
       <c r="I157" s="6" t="inlineStr"/>
       <c r="J157" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K157" s="6" t="inlineStr"/>
-      <c r="L157" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K157" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S9)</t>
+        </is>
+      </c>
+      <c r="L157" s="6" t="inlineStr">
+        <is>
+          <t>4f45f15 + e73ab59 - El argumento de ambito del Art. 4 se incorpora, en el codigo y en la hoja de ruta, y se cita por lo que el articulo AFIRMA: acota el ambito a edificaciones. No se le hace decir que excluye expresamente a los puentes, porque no los nombra.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S14): tracker — los nueve cierres nuevos con su commit
Las quince filas que S14 cierra ya llevaban su evidencia; nueve de ellas
(NOR-VOC-01/02/03/04, NOR-PRO-05, NOR-PUE-13, MAT-O19, NOR-COH-03, SIS-B-09)
no tenian ningun commit citado porque nunca se habian tocado. Se les escribe
el de la sesion. Las otras seis ya arrastraban el suyo y se les anade el de
S14 detras.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqmPnvMVziqsRG41X2Tjkf
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -7020,7 +7020,7 @@
       </c>
       <c r="L88" s="6" t="inlineStr">
         <is>
-          <t>S14 — `TW` (tirante sobre el fondo de la salida, m) y `cota_TW` (cota absoluta, msnm) quedan declarados en constantes_normativas.HOMONIMIA_TW con lo que los separa -- cota_TW = cota_fondo_salida + TW -- y con la acotacion de la propia ficha: hoy la confusion no se puede ejercitar porque las cuatro filas del CSV traen cota_TW vacia, de modo que se declara como riesgo de nomenclatura y no como error demostrado. Lo imprime M11.bloque_homonimias en las dos plantillas.</t>
+          <t>27f0963 — `TW` (tirante sobre el fondo de la salida, m) y `cota_TW` (cota absoluta, msnm) quedan declarados en constantes_normativas.HOMONIMIA_TW con lo que los separa -- cota_TW = cota_fondo_salida + TW -- y con la acotacion de la propia ficha: hoy la confusion no se puede ejercitar porque las cuatro filas del CSV traen cota_TW vacia, de modo que se declara como riesgo de nomenclatura y no como error demostrado. Lo imprime M11.bloque_homonimias en las dos plantillas.</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="L89" s="6" t="inlineStr">
         <is>
-          <t>S14 — Los TRES sentidos de «recubrimiento» en HOMONIMIA_RECUBRIMIENTO: (a) altura de relleno de tierra; (b) recubrimiento de concreto sobre el acero (Manual Tabla 2.9.1.5.5.3-1); (c) el que faltaba, el REVESTIMIENTO metalico o bituminoso de la plancha, verificado contra el PDF del EG-2013 -- Tabla 507-02 «Recubrimiento en peso de zinc, de acuerdo al espesor del acero base», pag. impresa 971 (PDF 979), 610 a 915 g/m2 --, que es el que gobierna la proteccion del TMC en este ambiente. Se corrige ademas la afirmacion «no tienen ninguna relacion»: la fila que se citaba para decirlo ACOPLA (a) y (b) en su propio renglon. Lo que se sostiene es lo suficiente: son magnitudes distintas, con unidades distintas, y ninguna sustituye a la otra.</t>
+          <t>27f0963 — Los TRES sentidos de «recubrimiento» en HOMONIMIA_RECUBRIMIENTO: (a) altura de relleno de tierra; (b) recubrimiento de concreto sobre el acero (Manual Tabla 2.9.1.5.5.3-1); (c) el que faltaba, el REVESTIMIENTO metalico o bituminoso de la plancha, verificado contra el PDF del EG-2013 -- Tabla 507-02 «Recubrimiento en peso de zinc, de acuerdo al espesor del acero base», pag. impresa 971 (PDF 979), 610 a 915 g/m2 --, que es el que gobierna la proteccion del TMC en este ambiente. Se corrige ademas la afirmacion «no tienen ninguna relacion»: la fila que se citaba para decirlo ACOPLA (a) y (b) en su propio renglon. Lo que se sostiene es lo suficiente: son magnitudes distintas, con unidades distintas, y ninguna sustituye a la otra.</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="L90" s="6" t="inlineStr">
         <is>
-          <t>S14 — HOMONIMIA_LUZ declara que «luz» es un dato de ENTRADA que clasifica el cruce (6.0 m, num. 4.1.1.3.1 y 4.1.1.5.1) y el diametro un RESULTADO del catalogo. Comprobado en el codigo que NINGUN modulo convierte una en otra: la luz entra en la Fase 2 y no vuelve a aparecer en el dimensionamiento, de modo que la equivalencia que el Manual no define tampoco hace falta. Queda anotado que el num. 4.1.1.3.4 a) admite «su equivalente de otra seccion» y que esa equivalencia hay que declararla ANTES de ofrecer una seccion no circular.</t>
+          <t>27f0963 — HOMONIMIA_LUZ declara que «luz» es un dato de ENTRADA que clasifica el cruce (6.0 m, num. 4.1.1.3.1 y 4.1.1.5.1) y el diametro un RESULTADO del catalogo. Comprobado en el codigo que NINGUN modulo convierte una en otra: la luz entra en la Fase 2 y no vuelve a aparecer en el dimensionamiento, de modo que la equivalencia que el Manual no define tampoco hace falta. Queda anotado que el num. 4.1.1.3.4 a) admite «su equivalente de otra seccion» y que esa equivalencia hay que declararla ANTES de ofrecer una seccion no circular.</t>
         </is>
       </c>
     </row>
@@ -7766,7 +7766,7 @@
       </c>
       <c r="L101" s="6" t="inlineStr">
         <is>
-          <t>S14 — «Clase F» se desambigua con las TRES acepciones del corpus -- clase de sitio sismica, concreto EG-2013 Tabla 503-07 y acero ASTM A668 del propio Manual, pag. impresa 289 --, escritas UNA vez en constantes_normativas.HOMONIMIA_CLASE_F y renderizadas por `homonimia_como_texto` en los dos sitios que las imprimen: M9.condicion_normativa_cabezal (pegada a la cadena sismica, donde el lector se encuentra el termino) y el glosario nuevo M11.bloque_homonimias.</t>
+          <t>27f0963 — «Clase F» se desambigua con las TRES acepciones del corpus -- clase de sitio sismica, concreto EG-2013 Tabla 503-07 y acero ASTM A668 del propio Manual, pag. impresa 289 --, escritas UNA vez en constantes_normativas.HOMONIMIA_CLASE_F y renderizadas por `homonimia_como_texto` en los dos sitios que las imprimen: M9.condicion_normativa_cabezal (pegada a la cadena sismica, donde el lector se encuentra el termino) y el glosario nuevo M11.bloque_homonimias.</t>
         </is>
       </c>
     </row>
@@ -11488,7 +11488,7 @@
       </c>
       <c r="L170" s="6" t="inlineStr">
         <is>
-          <t>S14 — `_NORMA_PRODUCTO` del concreto pasa de «ASTM C76 / AASHTO M170» -- las versiones EN PULGADAS -- a «AASHTO M 170M-04 / ASTM C 76M-02 (metrica)», que es como se designa el documento que hay en normas/ y que su num. 1.2 declara «the metric counterpart of M 170» (verificado sobre el PDF). La de TMC pasa a la designacion DUAL «AASHTO M 36 / ASTM A760/A760M-10», que es la del registro, sin inventarle una metrica que la norma no separa. Corregido tambien el comentario de `modelos.Material.norma_producto`, que ponia las imperiales como ejemplo.</t>
+          <t>27f0963 — `_NORMA_PRODUCTO` del concreto pasa de «ASTM C76 / AASHTO M170» -- las versiones EN PULGADAS -- a «AASHTO M 170M-04 / ASTM C 76M-02 (metrica)», que es como se designa el documento que hay en normas/ y que su num. 1.2 declara «the metric counterpart of M 170» (verificado sobre el PDF). La de TMC pasa a la designacion DUAL «AASHTO M 36 / ASTM A760/A760M-10», que es la del registro, sin inventarle una metrica que la norma no separa. Corregido tambien el comentario de `modelos.Material.norma_producto`, que ponia las imperiales como ejemplo.</t>
         </is>
       </c>
     </row>
@@ -11542,7 +11542,7 @@
       </c>
       <c r="L171" s="6" t="inlineStr">
         <is>
-          <t>S14 — Verificado contra el PDF del Manual, pagina por pagina: el texto del num. 2.8.1.3.1.2c esta en la pag. impresa 272 (PDF 273), la Figura 2.8.1.3.1.2c-1 -- suelos COHESIVOS -- en la 273 (PDF 274) y la Figura 2.8.1.3.1.2c-2 -- suelos NO COHESIVOS -- en la 274 (PDF 275). El rango declarado, «pags. 272-273», dejaba fuera la segunda. Corregido en NUMERAL_ZAPATA_EN_TALUD y en la fuente del criterio 'N_cq_N_gammaq_meyerhof', las dos con la figura atribuida a su pagina y con cual aplica segun el tipo de suelo de fundacion.</t>
+          <t>27f0963 — Verificado contra el PDF del Manual, pagina por pagina: el texto del num. 2.8.1.3.1.2c esta en la pag. impresa 272 (PDF 273), la Figura 2.8.1.3.1.2c-1 -- suelos COHESIVOS -- en la 273 (PDF 274) y la Figura 2.8.1.3.1.2c-2 -- suelos NO COHESIVOS -- en la 274 (PDF 275). El rango declarado, «pags. 272-273», dejaba fuera la segunda. Corregido en NUMERAL_ZAPATA_EN_TALUD y en la fuente del criterio 'N_cq_N_gammaq_meyerhof', las dos con la figura atribuida a su pagina y con cual aplica segun el tipo de suelo de fundacion.</t>
         </is>
       </c>
     </row>
@@ -12826,7 +12826,7 @@
       </c>
       <c r="L195" s="6" t="inlineStr">
         <is>
-          <t>S14 — `KU_METRICO` pasa a `KU_SI`, con el sufijo que CLAUDE.md exige a toda constante empirica dependiente de unidades, y con el equivalente imperial nombrado y la razon de no usarlo: en el sistema ingles Ku vale 1.0 -- la fuente los imprime juntos, «Ku Unit conversion 1.0 (1.811 SI)» -- y usar el 1.0 en metrico es el error silencioso SIMETRICO al del 29 de K_FRICCION_SI. Renombrado en sus cuatro consumidores y en el manifiesto; la hoja de ruta llevaba el nombre viejo en su Anexo B y se corrigio ahi tambien. La otra mitad de la ficha, el ambito de DIAMETRO_MIN, ya estaba cerrada en DIAMETRO_MIN_AMBITO con sus dos condicionantes.</t>
+          <t>27f0963 — `KU_METRICO` pasa a `KU_SI`, con el sufijo que CLAUDE.md exige a toda constante empirica dependiente de unidades, y con el equivalente imperial nombrado y la razon de no usarlo: en el sistema ingles Ku vale 1.0 -- la fuente los imprime juntos, «Ku Unit conversion 1.0 (1.811 SI)» -- y usar el 1.0 en metrico es el error silencioso SIMETRICO al del 29 de K_FRICCION_SI. Renombrado en sus cuatro consumidores y en el manifiesto; la hoja de ruta llevaba el nombre viejo en su Anexo B y se corrigio ahi tambien. La otra mitad de la ficha, el ambito de DIAMETRO_MIN, ya estaba cerrada en DIAMETRO_MIN_AMBITO con sus dos condicionantes.</t>
         </is>
       </c>
     </row>
@@ -12880,7 +12880,7 @@
       </c>
       <c r="L196" s="6" t="inlineStr">
         <is>
-          <t>S14 — Las cuatro referencias por NUMERO DE LINEA a la hoja de ruta que quedaban en el codigo se reanclaron por simbolo y texto, que es la regla 4 de CLAUDE.md: «linea 806» apuntaba a la longitud maxima de cuneta y ahora cita el comentario de la asignacion `D_MAX`; «linea 523» y «linea 546» caian en separadores «---» y ahora citan «tabla de Sec. 7.A, fila Concreto y TMC» y «tabla de Fase 8, fila TMC»; «linea 832» ahora cita el comentario de `H_RELLENO_MIN["tmc"]`. El defecto que la ficha denunciaba en el comentario de K_FRICCION_SI ya se habia corregido antes. De paso se reanclaron por simbolo siete referencias rotas del manifiesto (NUMERAL_C_PHI, NUMERAL_ZAPATA_TALUD_E050, Ks, NUMERAL_CRITICO, PERFIL_SUELO_PRESUNTO y los tres nombres inexistentes e3_/e4_/e5_, que son hoy `verificar_deslizamiento`, `verificar_estabilidad_global` y `verificar_talud`).</t>
+          <t>27f0963 — Las cuatro referencias por NUMERO DE LINEA a la hoja de ruta que quedaban en el codigo se reanclaron por simbolo y texto, que es la regla 4 de CLAUDE.md: «linea 806» apuntaba a la longitud maxima de cuneta y ahora cita el comentario de la asignacion `D_MAX`; «linea 523» y «linea 546» caian en separadores «---» y ahora citan «tabla de Sec. 7.A, fila Concreto y TMC» y «tabla de Fase 8, fila TMC»; «linea 832» ahora cita el comentario de `H_RELLENO_MIN["tmc"]`. El defecto que la ficha denunciaba en el comentario de K_FRICCION_SI ya se habia corregido antes. De paso se reanclaron por simbolo siete referencias rotas del manifiesto (NUMERAL_C_PHI, NUMERAL_ZAPATA_TALUD_E050, Ks, NUMERAL_CRITICO, PERFIL_SUELO_PRESUNTO y los tres nombres inexistentes e3_/e4_/e5_, que son hoy `verificar_deslizamiento`, `verificar_estabilidad_global` y `verificar_talud`).</t>
         </is>
       </c>
     </row>
@@ -13466,7 +13466,7 @@
       </c>
       <c r="L207" s="6" t="inlineStr">
         <is>
-          <t>S14 — Las constantes NUMERAL_* de modulo sin lector son OCHO, no siete, y su decision queda escrita una sola vez en `modelos.NUMERALES_DE_SECCION_SIN_LECTOR` -- junto a `ReferenciaNormativa`, que es la clase que define la distincion de la que se trata: son coordenadas del apartado de la hoja de ruta, no citas. Se dice por que no se borran (son el mapa modulo -&gt; apartado), por que NO se imprimen (meter «4.1» en una memoria como si fuera un numeral es el defecto que ReferenciaNormativa existe para impedir) y la segunda razon de dos de ellas, NUMERAL_V5 y NUMERAL_V8, que son bloqueos ya declarados. La guardia que lo vigile es trabajo de S16: escribir hoy un test contra el estado actual congelaria defectos que las fases de correccion siguen cerrando (regla 6 de CLAUDE.md).</t>
+          <t>27f0963 — Las constantes NUMERAL_* de modulo sin lector son OCHO, no siete, y su decision queda escrita una sola vez en `modelos.NUMERALES_DE_SECCION_SIN_LECTOR` -- junto a `ReferenciaNormativa`, que es la clase que define la distincion de la que se trata: son coordenadas del apartado de la hoja de ruta, no citas. Se dice por que no se borran (son el mapa modulo -&gt; apartado), por que NO se imprimen (meter «4.1» en una memoria como si fuera un numeral es el defecto que ReferenciaNormativa existe para impedir) y la segunda razon de dos de ellas, NUMERAL_V5 y NUMERAL_V8, que son bloqueos ya declarados. La guardia que lo vigile es trabajo de S16: escribir hoy un test contra el estado actual congelaria defectos que las fases de correccion siguen cerrando (regla 6 de CLAUDE.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S15): tracker — SIS-D-09 cerrado con su commit
Los otros tres IDs de la tarea ya estaban cerrados y se verificaron sobre el
codigo, no sobre el tracker: SIS-D-07 (cli.py vuelca
`criterios_con_verificacion_pendiente()` como hermano de
`trazabilidad_incompleta`), SIS-D-08 (ya no hay ningun [A] con valor y sin
sensibilidad: `clase_sitio` es [S] desde S13) y SIS-D-12 (la §14 del
manifiesto de citas declara que `v_max_hdpe` y `v_max_tmc` son cita cerrada y
no vacio agotado, que es el caso distinto).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SZRpYos6gGLbbuENkhbSaU
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -12504,11 +12504,19 @@
       <c r="I189" s="6" t="inlineStr"/>
       <c r="J189" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K189" s="6" t="inlineStr"/>
-      <c r="L189" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K189" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S15)</t>
+        </is>
+      </c>
+      <c r="L189" s="6" t="inlineStr">
+        <is>
+          <t>d158496 — la guardia que faltaba: DatoSitio.__post_init__ + _coherencia_de_datos_sitio() al importar, homologas de _verificar_criterio/_coherencia_de_etiquetas. Rechaza el caso exacto del hallazgo (trazabilidad="" con etiqueta="A") y los campos con que un [S] se reproduce. Va en __post_init__ y no solo en el barrido porque datos_sitio.py no tiene API de escritura: el unico camino es construir el objeto. tests/test_datos_sitio.py, 11 tests nuevos.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S16): tracker — 43 hallazgos de C09 y C10 marcados contra 52c11d2
Hoja `Hallazgos`: Estado / Responsable / Commit para los 43 IDs de la sesion
(40 Cerrado, 3 Cerrado parcial). Va en un commit aparte porque la columna
Commit cita el SHA del commit de codigo, que no puede contenerse a si mismo.

C09 y C10 quedan sin pendientes. Los 15 pendientes que restan en la matriz son
C14 (14) y C02 (1), que son sesiones posteriores.

Los tres parciales, y hasta donde llegan:
  SIS-F-01  se cubre el CONTRATO de la GUI, no sus 584 sentencias.
  SIS-F-13  M7 y M9 pasan a consumir caso patron; M2, M8 y M10 siguen sin el,
            porque fabricarles dorados aqui seria inventar el valor de
            referencia — justo lo que prohibe el conflicto n.7.
  MAT-O18   cerrados el contrato None de M3 y la asintota de M7; queda fuera
            la parte de R^(4/3).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JZjUKF26GeaqKXdZtUnT9Y
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -8886,11 +8886,19 @@
       <c r="I120" s="6" t="inlineStr"/>
       <c r="J120" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K120" s="6" t="inlineStr"/>
-      <c r="L120" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K120" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L120" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El manejador de EJECUTAR pasa de (OSError, ValueError) a (OSError, UnicodeDecodeError, json.JSONDecodeError), el mismo brazo estrecho que usa cli.py::main: un ValueError nacido en el pipeline ya no se muestra como 'No se pudo leer la entrada' ni se come el brazo que imprime la traza. UnicodeDecodeError se nombra explicitamente porque es subclase de ValueError y estrechar sin el habria sido una regresion. tests/test_gui_contrato.py.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
@@ -8936,11 +8944,19 @@
       <c r="I121" s="6" t="inlineStr"/>
       <c r="J121" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K121" s="6" t="inlineStr"/>
-      <c r="L121" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K121" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L121" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — PARCIAL Y DECLARADO COMO TAL en el encabezado de tests/test_gui_contrato.py (19 tests): se cubre el CONTRATO, no las 584 sentencias. Parte AST: forma de los brazos de excepcion, todos los manejadores y no solo el primero, BaseException prohibida, print_exc como sentencia directa del cuerpo. Parte EJECUTABLE con un doble de tkinter inyectado en sys.modules: _interpretar_valor_declarado y _leer_banderas, las dos reimplementaciones que la ficha nombra, mas la divergencia deliberada GUI-vs-CLI sobre '1,5', fijada como tal. Queda fuera el resto del cableado de widgets.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -8986,11 +9002,19 @@
       <c r="I122" s="6" t="inlineStr"/>
       <c r="J122" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K122" s="6" t="inlineStr"/>
-      <c r="L122" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K122" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L122" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La rama que SI escribe el archivo fuente de los criterios se ejecuta ahora sobre una copia del archivo en tmp_path, con lectura posterior del contenido escrito. tests/test_criterios_adoptados.py.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
@@ -9036,11 +9060,19 @@
       <c r="I123" s="6" t="inlineStr"/>
       <c r="J123" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K123" s="6" t="inlineStr"/>
-      <c r="L123" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K123" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L123" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Caso patron CP-9 nuevo (CP9_MONONOBE_OKABE, tres juegos con phi, i, beta, delta, k_h y k_v todos distintos y distintos de cero, mas CP9_RANKINE_LIMITE), autoverificado en el bloque __main__ del fixture con recomputacion independiente. El caso limite de Rankine era ciego a los signos porque con i=beta=delta=0 los cuatro cosenos son simetricos. Barrido de mutacion: los diez mutantes de signo de k_ae_mononobe_okabe y angulo_inercia_sismica MUEREN, incluido el [1+R]-&gt;[1-R] de la errata del Manual.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -9086,11 +9118,19 @@
       <c r="I124" s="6" t="inlineStr"/>
       <c r="J124" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K124" s="6" t="inlineStr"/>
-      <c r="L124" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K124" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L124" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Caso patron CP-9 bloque de empujes (CP9_EMPUJE_TRASDOS), con k_v = 0.15 de PRUEBA para que el factor (1-k_v) sea visible -- el test viejo invocaba con k_v = 0.0 y el mutante era indetectable por construccion. El unico assert era tautologico porque incremento_sismico llama a las mismas dos funciones que el test usaba para armar el lado derecho. Barrido de mutacion: los cuatro mutantes de empuje_activo_sismico_total mueren, mas los de empuje_activo_estatico y brazo_incremento_sismico.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
@@ -9136,11 +9176,19 @@
       <c r="I125" s="6" t="inlineStr"/>
       <c r="J125" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K125" s="6" t="inlineStr"/>
-      <c r="L125" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K125" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L125" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Asserts de VALOR sobre el FS de E3: verificar_deslizamiento se contrasta contra un FS calculado a mano (65/50 = 1.30), de modo que el mutante FS = R*A (4500) y la guarda invertida (fs = inf siempre) mueren los dos. Se abrio ademas, sin ID de auditoria propio, la contraparte que la ficha daba por cubierta. tests/test_M9_cabezal.py.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -9186,11 +9234,19 @@
       <c r="I126" s="6" t="inlineStr"/>
       <c r="J126" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K126" s="6" t="inlineStr"/>
-      <c r="L126" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K126" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L126" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — tests/test_modelos.py pasa de comparar ORDEN a comparar VALOR en EmpujesTrasdos.empuje_horizontal_total y .momento_volcante, con los terminos desglosados. Mueren * -&gt; /, + -&gt; -, borrar LS o WA de la suma, meter U_subpresion (que es vertical) en la horizontal y usar altura_empuje en vez de z_activo. Ademas modelos.EmpujesTrasdos.__post_init__ hace imposible el estado EQ a medias -- incremento_sismico con z_incremento=None contaba EQ en la fuerza y lo perdia en el momento volcante, que es NO conservador.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
@@ -9236,11 +9292,19 @@
       <c r="I127" s="6" t="inlineStr"/>
       <c r="J127" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K127" s="6" t="inlineStr"/>
-      <c r="L127" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K127" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L127" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Caso patron CP9_GEOMETRIA_7B, consumido por tests/test_M7_geometria.py, con assert de valor sobre la rama viva de longitud y proyeccion. Mueren los tres mutantes de la ficha y los cuatro mas que el barrido encontro en las mismas tres lineas, mas los dos de g2_cota_salida que ninguna auditoria habia reportado. Las referencias archivo:linea de la ficha (442/454/532/534) estaban corridas ~180 lineas; el cierre se ancla por simbolo.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -9286,11 +9350,19 @@
       </c>
       <c r="J128" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K128" s="6" t="inlineStr"/>
-      <c r="L128" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K128" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L128" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Cerrado con SIS-C-06: el barrido recorre cli.py y gui/app.py, con la regla estrechada de la capa de presentacion declarada en el encabezado de tests/test_sin_literales.py.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -9336,11 +9408,19 @@
       <c r="I129" s="6" t="inlineStr"/>
       <c r="J129" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K129" s="6" t="inlineStr"/>
-      <c r="L129" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K129" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L129" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La guardia de subcadena de factor_muro pasa a comprobacion AST (tests/apoyo/estructura.py::constructor_de_clave): no mira comillas, de modo que la entrada con comillas simples que evadia la version anterior ya no evade. Al portarla se descubrio que el test hermano estaba VERDE SOBRE UN COMENTARIO: FACTOR_MURO_TABLA se habia retirado de constantes_normativas.py (NOR-PUE-07) y la cadena sobrevivia dentro del comentario que explica la retirada. Reescrito contra los simbolos que si existen (REDUCCION_KH_POR_DESPLAZAMIENTO, FACTOR_MURO_DECLARACIONES).</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -9386,11 +9466,19 @@
       <c r="I130" s="6" t="inlineStr"/>
       <c r="J130" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K130" s="6" t="inlineStr"/>
-      <c r="L130" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K130" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L130" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Los 22 asserts de subcadena sobre el texto fuente pasan al AST (tests/apoyo/estructura.py: nombres_asignados, valor_asignado, nombres_usados, claves_de_dict, constructor_de_clave, llamadas_a, argumentos_de_texto). Un comentario o un docstring ya no los satisface. Afectados: test_sin_literales.py, test_criterios_adoptados.py, test_datos_sitio.py, test_M8_estructural.py.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
@@ -9436,11 +9524,19 @@
       <c r="I131" s="6" t="inlineStr"/>
       <c r="J131" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K131" s="6" t="inlineStr"/>
-      <c r="L131" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K131" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L131" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La marca deja de buscarse como subcadena de la linea y se detecta con tokenize, como COMMENT token: una marca dentro de un string o de un docstring ya no exime nada. Se exige ademas la razon ('# literal-ok: &lt;razon&gt;' con texto detras), como escribe CLAUDE.md; dos marcas del arbol que no la traian la llevan ahora. tests/test_sin_literales.py::test_sis_c_03_* y ::test_toda_marca_declara_su_razon.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -9486,11 +9582,19 @@
       <c r="I132" s="6" t="inlineStr"/>
       <c r="J132" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K132" s="6" t="inlineStr"/>
-      <c r="L132" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K132" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L132" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — _nodos_de_indice deja de eximir la CLAVE de una tabla declarada: un entero dentro de un subscript sobre un nombre en MAYUSCULAS es una magnitud, no una posicion, y cae. _base_del_subscript resuelve la raiz, de modo que TABLA[900][2500] cae en los dos niveles y no solo en el primero. El indice sobre una secuencia sigue exento, que es lo unico que CLAUDE.md permite.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
@@ -9536,11 +9640,19 @@
       <c r="I133" s="6" t="inlineStr"/>
       <c r="J133" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K133" s="6" t="inlineStr"/>
-      <c r="L133" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K133" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L133" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La lista de exentos se compara por RUTA RELATIVA a la raiz del barrido y no por nombre de archivo: un src/modulos/dominios.py ya no queda exento por homonimia. tests/test_sin_literales.py::test_sis_c_05_el_exento_se_reconoce_por_ruta_y_no_por_nombre.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -9590,11 +9702,19 @@
       </c>
       <c r="J134" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K134" s="6" t="inlineStr"/>
-      <c r="L134" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K134" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L134" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — cli.py, gui/app.py y verificar_sesion.py entran al barrido con una regla ESTRECHADA y declarada, homologa a la que ya tenia src/normativa/: un entero dentro de una llamada de presentacion pasa; un float o un complejo cae SIEMPRE, tambien marcado; una clave de tabla cae aunque este dentro de la llamada; lo demas cae salvo marca. Se anadieron 34 marcas de geometria y se nombraron ANCHO, SANGRIA_DETALLE, DECIMALES_PENDIENTE, HALLAZGOS_EN_LA_MATRIZ y ANCHO_CONSOLA. Ademas test_ningun_py_fuera_de_src_se_queda_sin_declarar cierra la FAMILIA: todo .py fuera de src/ tiene que estar vigilado o exento con su razon escrita (conftest.py es el unico exento, y su razon esta escrita).</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -9640,11 +9760,19 @@
       <c r="I135" s="6" t="inlineStr"/>
       <c r="J135" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K135" s="6" t="inlineStr"/>
-      <c r="L135" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K135" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L135" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La marca vale SOLO en la linea fisica del literal: una marca en linea propia ya no blanquea la linea siguiente. Las expresiones partidas de src/ que dependian de la linea anterior llevan ahora la marca en su propia linea. tests/test_sin_literales.py::test_sis_c_07_la_marca_en_linea_propia_no_exime_la_siguiente y ::test_sis_c_07_la_marca_al_final_de_la_linea_si_exime.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
@@ -9690,11 +9818,19 @@
       <c r="I136" s="6" t="inlineStr"/>
       <c r="J136" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K136" s="6" t="inlineStr"/>
-      <c r="L136" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K136" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L136" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La rama if informe.dimensionado de M11.exportar_csv se ejercita ahora con un punto REALMENTE dimensionado, comprobando las filas y no solo la cabecera. tests/test_cli.py.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
@@ -9740,11 +9876,19 @@
       <c r="I137" s="6" t="inlineStr"/>
       <c r="J137" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K137" s="6" t="inlineStr"/>
-      <c r="L137" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K137" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L137" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las guardas de ErrorProyecto sin cobertura quedan ejercitadas en M1, M2, M4, M5, M7, M9, criterios_adoptados, datos_sitio, modelos y cli. MEDIDO con coverage sobre el arbol de cierre: de los 115 `raise` de la taxonomia que hay en src/ + cli.py, 112 quedan cubiertos y solo 3 no, y esos tres son guardas defensivas provablemente inalcanzables del mismo tipo que documenta SIS-B-23 -- M1_clasificacion._categoria (segundo `raise`, tras un CategoriaTR() que ya tuvo exito), M9_cabezal:541 (fin del barrido de tramos que cubren todo el rango, con la razon escrita en el propio codigo) y M9_cabezal:1249 (idem para la tabla de h_eq). CORRECCION A LA FICHA: dice trece `raise` sin cobertura; la auditoria corrio sobre un arbol menor y el conteo no es portable al de hoy.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -9790,11 +9934,19 @@
       <c r="I138" s="6" t="inlineStr"/>
       <c r="J138" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K138" s="6" t="inlineStr"/>
-      <c r="L138" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K138" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L138" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las seis banderas del CLI sin cobertura (--pdf, --csv-resumen, --criterios y las tres restantes) se ejercitan de punta a punta, cableado bandera-&gt;funcion incluido. tests/test_cli.py.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
@@ -9840,11 +9992,19 @@
       <c r="I139" s="6" t="inlineStr"/>
       <c r="J139" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K139" s="6" t="inlineStr"/>
-      <c r="L139" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K139" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L139" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las dos ramas de _texto -- columna ausente del encabezado y celda de texto vacia (id, progresiva_km, familia, sucs_fundacion) -- se ejecutan y distinguen DatoFaltanteError de DatoInvalidoError. tests/test_M0_carga.py.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -9890,11 +10050,19 @@
       <c r="I140" s="6" t="inlineStr"/>
       <c r="J140" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K140" s="6" t="inlineStr"/>
-      <c r="L140" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K140" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L140" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — PARCIAL. El fixture gana CP-9 y con el pasan a consumir caso patron M7 (CP9_GEOMETRIA_7B) y M9 (CP9_MONONOBE_OKABE, CP9_RANKINE_LIMITE, CP9_EMPUJE_TRASDOS). SIGUEN SIN CASO PATRON M2, M8 y M10: para esos el fixture no da dorados y fabricarlos aqui seria inventar el valor de referencia, que es justo lo que el conflicto n.7 (CP-1 dorados / SIS-F-14) prohibe. Queda declarado como deuda abierta.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
@@ -10002,11 +10170,19 @@
       <c r="I142" s="6" t="inlineStr"/>
       <c r="J142" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K142" s="6" t="inlineStr"/>
-      <c r="L142" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K142" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L142" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las cinco afirmaciones falsas de los dos .md de fixtures se corrigen EN SU SITIO y con la razon, en vez de borrarse: v_max_hdpe y v_max_tmc ya no son vacios (4.572 m/s [C], WSDOT M 23-03.12 Tabla 8-4) y el fixture avisa de que aplicar 6.0/4.5 pisaria un valor con cita; remanso_derecho_via ya no aborta la corrida; los cinco sitios de AssertionError se anclan por SIMBOLO y no por archivo:linea (uno de los cinco ya no existe); Material.v_max_rango es un simbolo retirado; y el baseline de 653 tests se sustituye por la instruccion de leerlo de origin/main. Guardianes en tests/test_guardias_de_la_suite.py para que las afirmaciones no vuelvan a caducar en silencio.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
@@ -10052,11 +10228,19 @@
       <c r="I143" s="6" t="inlineStr"/>
       <c r="J143" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K143" s="6" t="inlineStr"/>
-      <c r="L143" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K143" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L143" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Los asserts se convierten a pytest.approx con tolerancia NOMBRADA (tests/apoyo/aproximacion.py: REL_TRANSPORTE para un valor que el pipeline solo transporta, ABS_CERO para la comparacion contra cero, donde la tolerancia relativa no existe). Guardian nuevo tests/test_guardias_de_la_suite.py::test_ningun_assert_compara_floats_con_igualdad_exacta, detector AST propio (==, !=, in, not in; contenedores; negativos; marca '# float-exacto: &lt;razon&gt;'), con su banco de casos y sus limites declarados. CORRECCION A LA FICHA: los 15 son el conteo del grep, que solo ve 'assert &lt;algo&gt; == &lt;literal float&gt;'; el detector AST encuentra ~57 con la definicion ancha, y todos los reales quedaron convertidos.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -10102,11 +10286,19 @@
       <c r="I144" s="6" t="inlineStr"/>
       <c r="J144" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K144" s="6" t="inlineStr"/>
-      <c r="L144" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K144" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L144" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El test que no invocaba codigo de produccion (reescribia la formula y se comparaba consigo mismo) pasa a llamar la funcion real; la autoverificacion de la formula queda donde corresponde, en el bloque __main__ de casos_patron.py. tests/test_M3_hidraulica.py.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
@@ -10214,11 +10406,19 @@
       <c r="I146" s="6" t="inlineStr"/>
       <c r="J146" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K146" s="6" t="inlineStr"/>
-      <c r="L146" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K146" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L146" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — La pertenencia a NUMEROS_PERMITIDOS se comprueba por TIPO ademas de por valor: un complejo cae siempre, tambien 0j y 2+0j, que se colaban porque son iguales a 0 y a 2. tests/test_sin_literales.py::test_sis_c_08_un_complejo_nunca_esta_permitido.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
@@ -10264,11 +10464,19 @@
       <c r="I147" s="6" t="inlineStr"/>
       <c r="J147" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K147" s="6" t="inlineStr"/>
-      <c r="L147" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K147" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L147" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Se detectan las conversiones desde texto (int, float, complex, Decimal, Fraction) con argumento literal que parsea como numero: int('500') y float('4.6') dejan de ser invisibles. tests/test_sin_literales.py::test_sis_c_09_*.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -10314,11 +10522,19 @@
       <c r="I148" s="6" t="inlineStr"/>
       <c r="J148" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K148" s="6" t="inlineStr"/>
-      <c r="L148" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K148" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L148" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las plantillas src/plantillas/*.html entran con su propia regla, declarada: fuera de los bloques &lt;style&gt; los unicos numeros admitidos son la numeracion de secciones de la memoria, porque toda magnitud entra por un marcador %%...%% que rellena M11. tests/test_sin_literales.py::test_las_plantillas_no_traen_valores_de_calculo.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
@@ -10364,11 +10580,19 @@
       <c r="I149" s="6" t="inlineStr"/>
       <c r="J149" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K149" s="6" t="inlineStr"/>
-      <c r="L149" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K149" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L149" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — M11.tableros_pendientes fallaba de forma ruidosa solo ante la perdida TOTAL del bloque; medido, retirar la tabla de un solo Tablero daba 2 tableros / 10 filas en vez de 3 / 15, en silencio. Ahora falla tambien ante la degradacion PARCIAL: una cabecera 'Tablero N' que no produce tabla, o un tablero con cero filas. tests/test_M11_reporte.py.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
@@ -10414,11 +10638,19 @@
       <c r="I150" s="6" t="inlineStr"/>
       <c r="J150" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K150" s="6" t="inlineStr"/>
-      <c r="L150" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K150" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L150" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El patron de escribir_valor_en_archivo se ejercita sobre los criterios de VALOR MULTILINEA y su ValueError queda cubierto. CORRECCION A LA FICHA: dice dos criterios de valor multilinea; medidos sobre el arbol de hoy son seis. tests/test_criterios_adoptados.py.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
@@ -10464,11 +10696,19 @@
       <c r="I151" s="6" t="inlineStr"/>
       <c r="J151" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K151" s="6" t="inlineStr"/>
-      <c r="L151" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K151" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L151" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las dos ramas de ImportError de MD quedan cubiertas sin borrar el modulo: la primera con un None en el registro, la segunda con un modulo presente que no expone verificar. Cubierta ademas la segunda deuda de la ficha, la resolucion del lote en disenar_lote. El skip permanente sigue siendo uno y sigue documentado. tests/test_MD.py.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
@@ -10514,11 +10754,19 @@
       <c r="I152" s="6" t="inlineStr"/>
       <c r="J152" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K152" s="6" t="inlineStr"/>
-      <c r="L152" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K152" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L152" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El borde de TOL_UMBRAL_NORMATIVO en _verificacion_por_fs se cubre con los tres casos que lo fijan (justo dentro, justo fuera, y el signo de la resta), de modo que invertir el signo de la tolerancia ya no deja la suite verde. tests/test_M9_cabezal.py.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
@@ -11698,11 +11946,19 @@
       <c r="I174" s="6" t="inlineStr"/>
       <c r="J174" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K174" s="6" t="inlineStr"/>
-      <c r="L174" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K174" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L174" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — cli._bloqueo dejaba de resolver toda clave con ca.criterio(): un [S] de corredor pendiente salia como KeyError, fallo de programa. Se anade criterios_adoptados.declaracion_de(clave), que resuelve indistintamente un criterio o un dato de sitio y devuelve la declaracion, y _bloqueo la consume. tests/test_cli.py.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
@@ -11922,11 +12178,19 @@
       <c r="I178" s="6" t="inlineStr"/>
       <c r="J178" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K178" s="6" t="inlineStr"/>
-      <c r="L178" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K178" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L178" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El diagnostico de Familia C que MD escribio es inalcanzable desde el CSV porque gana antes DatoFaltanteError('Q_m3s'): el hecho se fija con la fila C-01 del CSV de ejemplo y la rama se alcanza llamando _motivo_sin_candidatos directamente, con la razon de por que se hace asi escrita en el test. tests/test_MD.py.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
@@ -12620,11 +12884,19 @@
       <c r="I191" s="6" t="inlineStr"/>
       <c r="J191" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K191" s="6" t="inlineStr"/>
-      <c r="L191" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K191" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L191" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Los DatoInvalidoError que validan strings producidos por el propio codigo quedan declarados en M9_cabezal.py con la razon de por que la taxonomia del expediente es aqui la eleccion correcta y no un fallo de programa disfrazado. El quinto sitio que la ficha listaba, _recubrimiento_aashto_detallado, ya no existe.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="5" t="inlineStr">
@@ -12670,11 +12942,19 @@
       <c r="I192" s="6" t="inlineStr"/>
       <c r="J192" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K192" s="6" t="inlineStr"/>
-      <c r="L192" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K192" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L192" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — tr_desde_riesgo comprueba el DENOMINADOR antes de dividir y lanza DatoInvalidoError('R'): con R suficientemente pequeno (1-R)^(1/n) redondea a 1.0 y el ZeroDivisionError quedaba fuera de la taxonomia ErrorProyecto. Se comprueba el denominador, y en forma POSITIVA (if not denominador &gt; 0) para que nan tambien caiga, en vez de un umbral sobre R: el limite depende de n (R ~ n*eps/4, medido 1.39e-15 para n=25) y un umbral seria un literal de precision disfrazado de valor normativo. El mensaje nombra CRITERIO_RIESGO_PROPIETARIO, que es donde el revisor corrige. tests/test_M1_clasificacion.py.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="5" t="inlineStr">
@@ -12720,11 +13000,19 @@
       <c r="I193" s="6" t="inlineStr"/>
       <c r="J193" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K193" s="6" t="inlineStr"/>
-      <c r="L193" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K193" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L193" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — _a_float exige math.isfinite y lanza DatoInvalidoError: 'inf' pasa toda cota inferior y 'nan' es falso frente a &lt;= y a &gt;= a la vez, de modo que ninguna validacion de rango los atrapaba y el dato salia a la memoria como un numero que no lo es. Medido: inf SI se colaba por ocho columnas; nan no, y solo por suerte de redaccion. Se cierra ademas la simetria en criterios_adoptados y datos_sitio (_verificar_finitud, primero en el orden y absorbiendo OverflowError del entero enorme) y la via cli.py --declarar CLAVE=nan, que era el agujero mas grave: 'nan' e 'inf' son NOMBRES y no literales, ast.literal_eval los rechazaba y el respaldo de cadena guardaba el STRING por debajo de la guarda; M9_cabezal.cuantia_de_diseno hacia float() sobre el y la memoria salia con cuantia_adoptada = nan. tests/test_M0_carga.py, tests/test_cli.py, tests/test_criterios_adoptados.py, tests/test_datos_sitio.py.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="5" t="inlineStr">
@@ -12770,11 +13058,19 @@
       <c r="I194" s="6" t="inlineStr"/>
       <c r="J194" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K194" s="6" t="inlineStr"/>
-      <c r="L194" s="6" t="inlineStr"/>
+          <t>Cerrado parcial</t>
+        </is>
+      </c>
+      <c r="K194" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L194" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — PARCIAL. Se corrige el contrato de None de M3.tirante_normal, que mentia: None es CONSERVADOR, no literal; para D=0.90, S=0.005, n=0.013 se mide Q_pico=1.377 y Q_lleno=1.280, y en esa banda SI existe theta. Se declara ademas la asintota no acotada de M7.factor_esviaje. CORRECCION A LA FICHA: clasifica esos bordes como no alcanzables desde un CSV validado y DOS DE ELLOS SI LO SON -- esviaje ~89.999999 grados (factor 5.73e10) y la banda de None de M3. Queda fuera de este cierre la parte de R^(4/3) que la ficha lista aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="5" t="inlineStr">
@@ -13098,11 +13394,19 @@
       <c r="I200" s="6" t="inlineStr"/>
       <c r="J200" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K200" s="6" t="inlineStr"/>
-      <c r="L200" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K200" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L200" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las dos validaciones cruzadas que no son fila de la tabla de Sec. 1.5 -- diametro implicito y entrega por gravedad -- quedan declaradas en su punto de uso, en un bloque de M0_carga.py que dice que no vienen de la tabla y por que se aplican igual.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="5" t="inlineStr">
@@ -14012,11 +14316,19 @@
       <c r="I217" s="6" t="inlineStr"/>
       <c r="J217" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K217" s="6" t="inlineStr"/>
-      <c r="L217" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K217" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L217" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Las dos guardas provablemente inalcanzables (tabla de resguardo exhaustiva en M5.resguardo_por_cbr; esviaje negativo que M0 ya rechaza en M7.factor_esviaje) se cierran como corresponde a una guarda defensiva: no por inyeccion, sino con la DEMOSTRACION de que el dominio que M0 admite cae entero dentro del que la funcion admite, escrita en el test. Igual para la segunda guarda de M1._categoria. tests/test_M1_clasificacion.py, tests/test_M5_verificaciones.py, tests/test_M7_geometria.py.</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="5" t="inlineStr">
@@ -14228,11 +14540,19 @@
       <c r="I221" s="6" t="inlineStr"/>
       <c r="J221" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K221" s="6" t="inlineStr"/>
-      <c r="L221" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K221" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L221" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Los exportadores separan (OSError, ErrorProyecto) -- que el proyectista corrige y salen sin traza -- del fallo de programa, que imprime traceback.print_exc() como ya hacia el patron hermano de ejecutar_pipeline. CORRECCION A LA FICHA: dice tres exportadores; son CUATRO -- exportar_json estaba sin tocar y tambien se corrigio. tests/test_gui_contrato.py, con guardianes AST que impiden except BaseException, que revisan TODOS los brazos y no solo el primero, y que exigen print_exc como sentencia directa del cuerpo.</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="5" t="inlineStr">
@@ -14278,11 +14598,19 @@
       <c r="I222" s="6" t="inlineStr"/>
       <c r="J222" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K222" s="6" t="inlineStr"/>
-      <c r="L222" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K222" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L222" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — El unico raise de la GUI valida un campo TECLEADO por el usuario y se atrapa tres lineas mas abajo: es deliberado y no sale de la clase. Queda declarado en el docstring de _interpretar_valor_declarado y fijado por test, para que estrechar el brazo de captura no lo convierta en una traza. tests/test_gui_contrato.py.</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="5" t="inlineStr">
@@ -14328,11 +14656,19 @@
       <c r="I223" s="6" t="inlineStr"/>
       <c r="J223" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K223" s="6" t="inlineStr"/>
-      <c r="L223" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K223" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L223" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — establecer_valor_dinamico rechaza con ValueError, fuera de ErrorProyecto, y el docstring argumenta por que: CLAUDE.md define DatoInvalidoError para el dato del EXPEDIENTE, y una declaracion tecleada en la GUI no es un dato del expediente sino una entrada de interfaz que su propio manejador atrapa. tests/test_criterios_adoptados.py fija el contrato en los dos sentidos.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="5" t="inlineStr">
@@ -14378,11 +14714,19 @@
       <c r="I224" s="6" t="inlineStr"/>
       <c r="J224" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K224" s="6" t="inlineStr"/>
-      <c r="L224" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K224" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S16)</t>
+        </is>
+      </c>
+      <c r="L224" s="6" t="inlineStr">
+        <is>
+          <t>52c11d2 — Lo que faltaba era la actualizacion de la CONSTITUCION, como decia la propia ficha: CLAUDE.md ensancha la clausula de DatoFaltanteError para cubrir el dato que no viene del CSV (tablero externo), que es lo que modelos.py ya declaraba y el codigo ya explotaba. tests/test_criterios_adoptados.py.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S16.5): tracker — 5 hallazgos anclados contra 96084e8
Segundo commit de la sesion, por la misma razon que fa03f18 lo fue de S16: la
columna Commit no puede llevar el SHA del commit que la contiene. SIS-G-03 no
entra aqui porque queda declarado sin cerrar y no tiene commit que citar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016v7UEbDH9oPPpknmTudDGf
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -10093,7 +10093,7 @@
       <c r="L140" s="6" t="inlineStr">
         <is>
           <t>52c11d2 — PARCIAL. El fixture gana CP-9 y con el pasan a consumir caso patron M7 (CP9_GEOMETRIA_7B) y M9 (CP9_MONONOBE_OKABE, CP9_RANKINE_LIMITE, CP9_EMPUJE_TRASDOS). SIGUEN SIN CASO PATRON M2, M8 y M10: para esos el fixture no da dorados y fabricarlos aqui seria inventar el valor de referencia, que es justo lo que el conflicto n.7 (CP-1 dorados / SIS-F-14) prohibe. Queda declarado como deuda abierta.
-PRECISADO EN S16.5 (fase1) — pendiente de SHA (sin correccion de codigo; la frontera se describia de menos). Hoy son CINCO los tests que no importan casos_patron, no tres, y por TRES razones distintas que no se pueden contar juntas -- docs/linea_base.md ya avisaba en S1 que 'el grep real da 7 modulos, verificar alcance exacto en la fase de correccion':
+PRECISADO EN 96084e8 (fase1, S16.5) (sin correccion de codigo; la frontera se describia de menos). Hoy son CINCO los tests que no importan casos_patron, no tres, y por TRES razones distintas que no se pueden contar juntas -- docs/linea_base.md ya avisaba en S1 que 'el grep real da 7 modulos, verificar alcance exacto en la fase de correccion':
   * M2, M8, M10 — no hay dorado que traer sin violar el conflicto n.7. Es la unica deuda de las tres. QUE HARIA FALTA TRAER a cada uno queda escrito en la §15 del plan (hoja_de_ruta_correcciones_v12.md), con la fuente concreta: series de diametros nominales de las normas de producto para M2; AASHTO M 170M Tablas 1-5 y ASTM A796/A796M para M8; y para M10 no una norma sino el expediente vial (seccion de cuneta, su n, la intensidad de TR=35 y el metodo de area tributaria), porque su brazo normativo ya es [N] y un caso patron sobre el seria tautologico.
   * M5 — NO es deuda de dorado: el fixture SI define su caso (CP3_VELOCIDAD_MINIMA, Sec. 5.2), pero lo consumen test_M3 y test_constantes_normativas en vez de test_M5.
   * M11 — modulo de reporte, no de calculo: no le corresponde dorado numerico.</t>
@@ -13108,7 +13108,7 @@
       </c>
       <c r="L194" s="6" t="inlineStr">
         <is>
-          <t>52c11d2 (S16, parcial) + S16.5 (fase1) — pendiente de SHA (cierre). S16 corrigio el contrato de None de M3.tirante_normal y declaro la asintota de M7.factor_esviaje, y ya habia refutado la afirmacion de la ficha de que 'ninguno es alcanzable desde el CSV validado' en DOS de sus clausulas. S16.5 remide las CUATRO restantes, ninguna heredada:
+          <t>52c11d2 (S16, parcial) + 96084e8 (fase1, S16.5) (cierre). S16 corrigio el contrato de None de M3.tirante_normal y declaro la asintota de M7.factor_esviaje, y ya habia refutado la afirmacion de la ficha de que 'ninguno es alcanzable desde el CSV validado' en DOS de sus clausulas. S16.5 remide las CUATRO restantes, ninguna heredada:
 (1) R^(4/3) underflow (R&lt;=~1e-243): NO ALCANZABLE, con dos barreras independientes medidas. (a) Ningun Q en 325 decadas atraviesa tirante_critico con D=1e-243. (b) Aun inyectando `critico` a mano para saltarse esa guardia, control_salida revienta ANTES en _geometria_de_referencia (Q/A), porque A=pi*D^2/4 subdesborda 81 ordenes de magnitud antes que R^(4/3). Solo se alcanza llamando perdida_carga directamente con un R que no viene de ningun D. Se declara sin guardia.
 (2) q*^2 overflow (Q&gt;=~1.3e154): SI ALCANZABLE, Y LA FICHA LO ANCLA MAL. No esta en q*: esta en `Q ** 2` de _residuo_critico. Q_m3s no tiene techo en dominios.py, de modo que Q=1e155 llega entero desde un CSV valido y float.__pow__ lanza OverflowError CRUDO (Q=1e154 todavia cae como DatoInvalidoError por la guardia de bracket). CERRADO con guardia + test, con LimiteNumericoError. TERCERA correccion a la ficha.
 (3) 'las guardas de M-O nunca capturan psi=90 exacto': REFUTADA. k_v=1.0 da psi=90.0 y hoy dispara DisenoNoFactibleError.
@@ -14321,7 +14321,7 @@
       </c>
       <c r="L216" s="6" t="inlineStr">
         <is>
-          <t>S16.5 (fase1) — pendiente de SHA. LAS DOS AFIRMACIONES DE LA FICHA VERIFICADAS CONTRA EL CODIGO DE HOY, y la segunda se sostiene con MAS fuerza que cuando se escribio:
+          <t>96084e8 (fase1, S16.5). LAS DOS AFIRMACIONES DE LA FICHA VERIFICADAS CONTRA EL CODIGO DE HOY, y la segunda se sostiene con MAS fuerza que cuando se escribio:
 (a) aplica_sobrecarga_trasdos SI declara su motivo en su docstring, y ademas ya figura en M9.FUNCIONES_SIN_CONSUMIDOR con su razon escrita. Nada que hacer.
 (b) la acusacion sobre v_max_definida es falsa, y hoy mas: el simbolo en que se apoyaba, Material.v_max_rango, YA NO EXISTE en el repositorio (retirado al cerrar SIS-A-06). No hay nada que reimplementar porque no hay que reimplementar.
 Quedaban las DOS utilidades sin llamador de produccion, y se cierran escribiendo su decision en el docstring de cada una -- mismo tratamiento que la ficha ya acepto para aplica_sobrecarga_trasdos, y donde el revisor la busca: criterios_adoptados.limpiar_valores_dinamicos (una corrida de la CLI es un proceso de un solo uso y no necesita borrar todo; la GUI retira UNA clave; el consumidor real es conftest.py, que la nombra al explicar su fixture autouse) y M11_reporte.marcadores_de_la_memoria (puerta publica del contrato de la plantilla, para no atar a un consumidor externo al nombre de la constante MARCADORES). NO se crean dos registros FUNCIONES_SIN_CONSUMIDOR nuevos de una entrada cada uno.</t>
@@ -15400,7 +15400,7 @@
       </c>
       <c r="L236" s="6" t="inlineStr">
         <is>
-          <t>S16.5 (fase1) — pendiente de SHA. Declarado por S16 en el docstring de _verificar_finitud sin ID y sin cerrar; S16.5 lo da de alta y lo cierra. Guardia a la SALIDA de M7 (_exigir_finito), no a la entrada de dominios.py. Excepcion: modelos.LimiteNumericoError, quinta de la taxonomia (NO DatoInvalidoError: el dato cumple su rango, es la aritmetica la que no cabe). MEDIDO: cota_rasante=1e308 -&gt; altura_terraplen finita 1e308, proyeccion_taludes=inf. Barrido previo de los inf legitimos: son DOS (M9.verificar_volteo y M9.verificar_deslizamiento), la guardia vive solo en M7 y un test fija el censo. CLAUDE.md enmendada de cuatro excepciones a cinco</t>
+          <t>96084e8 (fase1, S16.5). Declarado por S16 en el docstring de _verificar_finitud sin ID y sin cerrar; S16.5 lo da de alta y lo cierra. Guardia a la SALIDA de M7 (_exigir_finito), no a la entrada de dominios.py. Excepcion: modelos.LimiteNumericoError, quinta de la taxonomia (NO DatoInvalidoError: el dato cumple su rango, es la aritmetica la que no cabe). MEDIDO: cota_rasante=1e308 -&gt; altura_terraplen finita 1e308, proyeccion_taludes=inf. Barrido previo de los inf legitimos: son DOS (M9.verificar_volteo y M9.verificar_deslizamiento), la guardia vive solo en M7 y un test fija el censo. CLAUDE.md enmendada de cuatro excepciones a cinco</t>
         </is>
       </c>
     </row>
@@ -15462,7 +15462,7 @@
       </c>
       <c r="L237" s="6" t="inlineStr">
         <is>
-          <t>S16.5 (fase1) — pendiente de SHA. Hallado al remedir MAT-O18. MEDIDO con D=0.90 m y CERO criterios declarados de mas: Q=1e-32 resuelve (theta=2.979e-08, area positiva), Q=1e-33 revienta. Umbral real: A=(D^2/8)(theta - sen theta) vale exactamente 0.0 desde theta&lt;=2.149e-08, porque theta-sen(theta)~theta^3/6 cae bajo el ultimo bit de theta. IRONIA UTIL: _residuo_critico YA esquiva esta misma cancelacion a proposito (por eso escribe A^3/T y no divide entre A^3) -- la defensa estaba en el residuo y faltaba tras el solver. Guardia con la FORMA de MAT-D13 (umbral medido, `not geom.A &gt; 0` en positivo para atrapar NaN, mensaje que nombra el par (Q,D)) y clase LimiteNumericoError</t>
+          <t>96084e8 (fase1, S16.5). Hallado al remedir MAT-O18. MEDIDO con D=0.90 m y CERO criterios declarados de mas: Q=1e-32 resuelve (theta=2.979e-08, area positiva), Q=1e-33 revienta. Umbral real: A=(D^2/8)(theta - sen theta) vale exactamente 0.0 desde theta&lt;=2.149e-08, porque theta-sen(theta)~theta^3/6 cae bajo el ultimo bit de theta. IRONIA UTIL: _residuo_critico YA esquiva esta misma cancelacion a proposito (por eso escribe A^3/T y no divide entre A^3) -- la defensa estaba en el residuo y faltaba tras el solver. Guardia con la FORMA de MAT-D13 (umbral medido, `not geom.A &gt; 0` en positivo para atrapar NaN, mensaje que nombra el par (Q,D)) y clase LimiteNumericoError</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S17): tracker — SIS-A-17, SIS-A-18 y SIS-A-10 cerrados contra 5ec63ae
SIS-F-01 sigue en «Cerrado parcial» y se anota lo que S17 le avanza: la
funcionalidad nueva nace con 86 tests ejecutables y con la comprobacion de
punta a punta que SIS-A-01 nunca tuvo. Lo que queda sin cubrir es el cableado
de widgets de gui/app.py anterior a esta sesion.

SIS-A-10 se cierra en sus DOS mitades --- las cuatro pestanas, incluida la que
reescribe criterios_adoptados.py, y el CSV en la lista de exportaciones ---,
que es lo que la ficha reprocha.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01276FPs6JzvFNmcC8EXPLMe
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -8981,12 +8981,12 @@
       </c>
       <c r="K121" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S16)</t>
+          <t>Claude Code (fase1, S16 + S17)</t>
         </is>
       </c>
       <c r="L121" s="6" t="inlineStr">
         <is>
-          <t>52c11d2 — PARCIAL Y DECLARADO COMO TAL en el encabezado de tests/test_gui_contrato.py (19 tests): se cubre el CONTRATO, no las 584 sentencias. Parte AST: forma de los brazos de excepcion, todos los manejadores y no solo el primero, BaseException prohibida, print_exc como sentencia directa del cuerpo. Parte EJECUTABLE con un doble de tkinter inyectado en sys.modules: _interpretar_valor_declarado y _leer_banderas, las dos reimplementaciones que la ficha nombra, mas la divergencia deliberada GUI-vs-CLI sobre '1,5', fijada como tal. Queda fuera el resto del cableado de widgets.</t>
+          <t>52c11d2 — PARCIAL Y DECLARADO COMO TAL en el encabezado de tests/test_gui_contrato.py (19 tests): se cubre el CONTRATO, no las 584 sentencias. Parte AST: forma de los brazos de excepcion, todos los manejadores y no solo el primero, BaseException prohibida, print_exc como sentencia directa del cuerpo. Parte EJECUTABLE con un doble de tkinter inyectado en sys.modules: _interpretar_valor_declarado y _leer_banderas, las dos reimplementaciones que la ficha nombra, mas la divergencia deliberada GUI-vs-CLI sobre '1,5', fijada como tal. Queda fuera el resto del cableado de widgets. || S17 (5ec63ae) — sigue PARCIAL y avanza mucho: la funcionalidad nueva de la GUI nace con 86 tests ejecutables (47 de contenido de la ventana, 33 del camino de declaracion, 6 de contrato) y con la comprobacion DE PUNTA A PUNTA que faltaba: declarar desde la ventana -&gt; pipeline -&gt; la memoria imprime el valor como declarado y con su procedencia. La estrategia que lo hace posible es partir el componente: el CONTENIDO vive en src/ventana_normativa.py y se compara campo a campo sin escritorio; gui/ventana_normativa.py solo cablea widgets. Sigue sin cubrirse el cableado de widgets de gui/app.py anterior a esta sesion.</t>
         </is>
       </c>
     </row>
@@ -12272,11 +12272,19 @@
       <c r="I179" s="6" t="inlineStr"/>
       <c r="J179" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K179" s="6" t="inlineStr"/>
-      <c r="L179" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K179" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S17)</t>
+        </is>
+      </c>
+      <c r="L179" s="6" t="inlineStr">
+        <is>
+          <t>5ec63ae — cerrado de paso al reescribir ese encabezado para SIS-A-17 y SIS-A-18, y en las DOS mitades que la ficha nombra: la lista dice ahora las cuatro pestanas --- incluida la de Criterios, que es la que reescribe criterios_adoptados.py y la que faltaba --- y la de exportaciones nombra el CSV junto a JSON, HTML y PDF.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="5" t="inlineStr">
@@ -13497,11 +13505,19 @@
       <c r="I201" s="6" t="inlineStr"/>
       <c r="J201" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K201" s="6" t="inlineStr"/>
-      <c r="L201" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K201" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S17)</t>
+        </is>
+      </c>
+      <c r="L201" s="6" t="inlineStr">
+        <is>
+          <t>5ec63ae — la pestana 1 expone el alcance de la corrida con las constantes ALCANCE_PERFIL/ALCANCE_EXPEDIENTE de cli.py (no dos cadenas escritas otra vez), el valor llega a cli.correr, y las dos exportaciones de memoria eligen plantilla con cli.plantilla_por_alcance --- la MISMA funcion que usa cli.main, para que la misma corrida no de dos memorias segun la puerta. memoria_perfil.html deja de ser inalcanzable desde la interfaz. El resumen anade dos filas: el alcance y el numero de etapas diferidas por el. Comprobado con Tk real bajo Xvfb: la corrida de perfil desde la ventana produce la memoria de perfil. Cuatro tests de contrato en tests/test_gui_contrato.py.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="5" t="inlineStr">
@@ -13547,11 +13563,19 @@
       <c r="I202" s="6" t="inlineStr"/>
       <c r="J202" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K202" s="6" t="inlineStr"/>
-      <c r="L202" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K202" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S17)</t>
+        </is>
+      </c>
+      <c r="L202" s="6" t="inlineStr">
+        <is>
+          <t>5ec63ae — la sesion (formato v2) guarda "alcance" y "criterios", y este ultimo lleva los valores dinamicos Y la procedencia de cada uno. Se restaura por declaracion.restaurar_sesion, que repone con establecer_valor_dinamico --- la misma guardia que el archivo ---, de modo que un JSON editado a mano no es una puerta de atras. Lo que la guardia rechaza NO se descarta en silencio: sale con su motivo en un aviso. Una sesion v1 se sigue leyendo y avisa de lo que no traia (patron de legacy/Tc.py). Tests: round-trip por json en tests/test_declaracion.py y contrato en tests/test_gui_contrato.py.</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S17): tracker — las tres filas citan ya su SHA de main
El PR #1 se reviso, se aprobo y se fusiono (6ff80fc). SIS-A-17, SIS-A-18 y
SIS-A-10 pasan de «PR abierto contra main, NO fusionado» a «Cerrado» y citan
5ec63ae, que desde la fusion es ancestro de main. A SIS-F-01 se le devuelve el
SHA: su anotacion de S17 decia «PR ABIERTO Y NO FUSIONADO --- nada de esto
esta en main todavia», y eso ya no es verdad.

Efecto en verificar_sesion.py, que es el que importa: las tres filas vuelven
al alcance del chequeo 4 («todo hallazgo cerrado cita un commit presente en
main»), que es donde tienen que estar. Mientras el trabajo no estaba en main,
quedarse fuera de ese chequeo era lo correcto; ahora lo correcto es lo
contrario.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01276FPs6JzvFNmcC8EXPLMe
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -8986,7 +8986,7 @@
       </c>
       <c r="L121" s="6" t="inlineStr">
         <is>
-          <t>52c11d2 — PARCIAL Y DECLARADO COMO TAL en el encabezado de tests/test_gui_contrato.py (19 tests): se cubre el CONTRATO, no las 584 sentencias. Parte AST: forma de los brazos de excepcion, todos los manejadores y no solo el primero, BaseException prohibida, print_exc como sentencia directa del cuerpo. Parte EJECUTABLE con un doble de tkinter inyectado en sys.modules: _interpretar_valor_declarado y _leer_banderas, las dos reimplementaciones que la ficha nombra, mas la divergencia deliberada GUI-vs-CLI sobre '1,5', fijada como tal. Queda fuera el resto del cableado de widgets. || S17 (rama claude/ventanas-emergentes-4-2-4-3-s50kk0, PR ABIERTO Y NO FUSIONADO --- nada de esto esta en main todavia): la funcionalidad nueva de la GUI nace con 86 tests ejecutables (47 de contenido de la ventana, 33 del camino de declaracion, 6 de contrato) y con la comprobacion DE PUNTA A PUNTA que faltaba: declarar desde la ventana -&gt; pipeline -&gt; la memoria imprime el valor como declarado y con su procedencia. La estrategia que lo hace posible es partir el componente: el CONTENIDO vive en src/ventana_normativa.py y se compara campo a campo sin escritorio; gui/ventana_normativa.py solo cablea widgets. Sigue sin cubrirse el cableado de widgets de gui/app.py anterior a esta sesion. Y EL CODIGO NUEVO TAMPOCO, dicho aqui para que no se lea de menos: gui/ventana_normativa.py --- el modulo de S17 que pinta widgets --- NO tiene cobertura automatica con Tk real. Se verifico UNA VEZ a mano, bajo Xvfb (las cuatro caras construidas sobre doce variables, la declaracion desde una fila, los tres colores del campo de rango al escribir y la corrida de perfil produciendo memoria_perfil.html), y esa comprobacion no quedo en la suite: no protege contra regresion. Lo que la suite si vigila de ese archivo es su ARBOL (brazos de excepcion, que recorra el orden visual declarado, que declare por declaracion.py y no por su cuenta) y, aparte, TODO su contenido a traves de src/ventana_normativa.py. Es el MISMO HUECO que la ficha declara para gui/app.py, no uno nuevo ni uno menor: el codigo que construye widgets sigue sin ejecutarse en la suite, y probarlo con un doble de tkinter seria un espejismo --- lo que se veria correr no es lo que corre en pantalla.</t>
+          <t>52c11d2 — PARCIAL Y DECLARADO COMO TAL en el encabezado de tests/test_gui_contrato.py (19 tests): se cubre el CONTRATO, no las 584 sentencias. Parte AST: forma de los brazos de excepcion, todos los manejadores y no solo el primero, BaseException prohibida, print_exc como sentencia directa del cuerpo. Parte EJECUTABLE con un doble de tkinter inyectado en sys.modules: _interpretar_valor_declarado y _leer_banderas, las dos reimplementaciones que la ficha nombra, mas la divergencia deliberada GUI-vs-CLI sobre '1,5', fijada como tal. Queda fuera el resto del cableado de widgets. || S17 (5ec63ae, fusionado en main por 6ff80fc): la funcionalidad nueva de la GUI nace con 86 tests ejecutables (47 de contenido de la ventana, 33 del camino de declaracion, 6 de contrato) y con la comprobacion DE PUNTA A PUNTA que faltaba: declarar desde la ventana -&gt; pipeline -&gt; la memoria imprime el valor como declarado y con su procedencia. La estrategia que lo hace posible es partir el componente: el CONTENIDO vive en src/ventana_normativa.py y se compara campo a campo sin escritorio; gui/ventana_normativa.py solo cablea widgets. Sigue sin cubrirse el cableado de widgets de gui/app.py anterior a esta sesion. Y EL CODIGO NUEVO TAMPOCO, dicho aqui para que no se lea de menos: gui/ventana_normativa.py --- el modulo de S17 que pinta widgets --- NO tiene cobertura automatica con Tk real. Se verifico UNA VEZ a mano, bajo Xvfb (las cuatro caras construidas sobre doce variables, la declaracion desde una fila, los tres colores del campo de rango al escribir y la corrida de perfil produciendo memoria_perfil.html), y esa comprobacion no quedo en la suite: no protege contra regresion. Lo que la suite si vigila de ese archivo es su ARBOL (brazos de excepcion, que recorra el orden visual declarado, que declare por declaracion.py y no por su cuenta) y, aparte, TODO su contenido a traves de src/ventana_normativa.py. Es el MISMO HUECO que la ficha declara para gui/app.py, no uno nuevo ni uno menor: el codigo que construye widgets sigue sin ejecutarse en la suite, y probarlo con un doble de tkinter seria un espejismo --- lo que se veria correr no es lo que corre en pantalla.</t>
         </is>
       </c>
     </row>
@@ -12272,7 +12272,7 @@
       <c r="I179" s="6" t="inlineStr"/>
       <c r="J179" s="6" t="inlineStr">
         <is>
-          <t>PR abierto contra main, NO fusionado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K179" s="6" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="L179" s="6" t="inlineStr">
         <is>
-          <t>NO FUSIONADO. El trabajo vive en la rama claude/ventanas-emergentes-4-2-4-3-s50kk0 (HEAD 4bfda57, con el cambio de codigo en su commit padre) y NO esta en main: hay un PR abierto, pendiente de revision. Esta fila NO dice «Cerrado» a proposito, y no cita ningun SHA de main porque no lo hay. Se pasa a «Cerrado», con el SHA de la fusion, cuando el PR se fusione. Cerrado de paso al reescribir el encabezado de gui/app.py para SIS-A-17 y SIS-A-18, y en las DOS mitades que la ficha nombra: la lista dice ahora las cuatro pestanas --- incluida la de Criterios, que es la que reescribe criterios_adoptados.py y la que faltaba --- y la de exportaciones nombra el CSV junto a JSON, HTML y PDF.</t>
+          <t>5ec63ae (fusionado en main por 6ff80fc, PR #1, revisado y aprobado). Cerrado de paso al reescribir el encabezado de gui/app.py para SIS-A-17 y SIS-A-18, y en las DOS mitades que la ficha nombra: la lista dice ahora las cuatro pestanas --- incluida la de Criterios, que es la que reescribe criterios_adoptados.py y la que faltaba --- y la de exportaciones nombra el CSV junto a JSON, HTML y PDF.</t>
         </is>
       </c>
     </row>
@@ -13505,7 +13505,7 @@
       <c r="I201" s="6" t="inlineStr"/>
       <c r="J201" s="6" t="inlineStr">
         <is>
-          <t>PR abierto contra main, NO fusionado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K201" s="6" t="inlineStr">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="L201" s="6" t="inlineStr">
         <is>
-          <t>NO FUSIONADO. El trabajo vive en la rama claude/ventanas-emergentes-4-2-4-3-s50kk0 (HEAD 4bfda57, con el cambio de codigo en su commit padre) y NO esta en main: hay un PR abierto, pendiente de revision. Esta fila NO dice «Cerrado» a proposito, y no cita ningun SHA de main porque no lo hay. Se pasa a «Cerrado», con el SHA de la fusion, cuando el PR se fusione. La pestana 1 expone el alcance de la corrida con las constantes ALCANCE_PERFIL/ALCANCE_EXPEDIENTE de cli.py (no dos cadenas escritas otra vez), el valor llega a cli.correr, y las dos exportaciones de memoria eligen plantilla con cli.plantilla_por_alcance --- la MISMA funcion que usa cli.main, para que la misma corrida no de dos memorias segun la puerta. memoria_perfil.html deja de ser inalcanzable desde la interfaz. El resumen anade dos filas: el alcance y el numero de etapas diferidas por el. Comprobado con Tk real bajo Xvfb: la corrida de perfil desde la ventana produce la memoria de perfil. Cuatro tests de contrato en tests/test_gui_contrato.py.</t>
+          <t>5ec63ae (fusionado en main por 6ff80fc, PR #1, revisado y aprobado). La pestana 1 expone el alcance de la corrida con las constantes ALCANCE_PERFIL/ALCANCE_EXPEDIENTE de cli.py (no dos cadenas escritas otra vez), el valor llega a cli.correr, y las dos exportaciones de memoria eligen plantilla con cli.plantilla_por_alcance --- la MISMA funcion que usa cli.main, para que la misma corrida no de dos memorias segun la puerta. memoria_perfil.html deja de ser inalcanzable desde la interfaz. El resumen anade dos filas: el alcance y el numero de etapas diferidas por el. Comprobado con Tk real bajo Xvfb: la corrida de perfil desde la ventana produce la memoria de perfil. Cuatro tests de contrato en tests/test_gui_contrato.py.</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
       <c r="I202" s="6" t="inlineStr"/>
       <c r="J202" s="6" t="inlineStr">
         <is>
-          <t>PR abierto contra main, NO fusionado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K202" s="6" t="inlineStr">
@@ -13573,7 +13573,7 @@
       </c>
       <c r="L202" s="6" t="inlineStr">
         <is>
-          <t>NO FUSIONADO. El trabajo vive en la rama claude/ventanas-emergentes-4-2-4-3-s50kk0 (HEAD 4bfda57, con el cambio de codigo en su commit padre) y NO esta en main: hay un PR abierto, pendiente de revision. Esta fila NO dice «Cerrado» a proposito, y no cita ningun SHA de main porque no lo hay. Se pasa a «Cerrado», con el SHA de la fusion, cuando el PR se fusione. La sesion (formato v2) guarda "alcance" y "criterios", y este ultimo lleva los valores dinamicos Y la procedencia de cada uno. Se restaura por declaracion.restaurar_sesion, que repone con establecer_valor_dinamico --- la misma guardia que el archivo ---, de modo que un JSON editado a mano no es una puerta de atras. Lo que la guardia rechaza NO se descarta en silencio: sale con su motivo en un aviso. Una sesion v1 se sigue leyendo y avisa de lo que no traia (patron de legacy/Tc.py). Tests: round-trip por json en tests/test_declaracion.py y contrato en tests/test_gui_contrato.py.</t>
+          <t>5ec63ae (fusionado en main por 6ff80fc, PR #1, revisado y aprobado). La sesion (formato v2) guarda "alcance" y "criterios", y este ultimo lleva los valores dinamicos Y la procedencia de cada uno. Se restaura por declaracion.restaurar_sesion, que repone con establecer_valor_dinamico --- la misma guardia que el archivo ---, de modo que un JSON editado a mano no es una puerta de atras. Lo que la guardia rechaza NO se descarta en silencio: sale con su motivo en un aviso. Una sesion v1 se sigue leyendo y avisa de lo que no traia (patron de legacy/Tc.py). Tests: round-trip por json en tests/test_declaracion.py y contrato en tests/test_gui_contrato.py.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S18): tracker — SIS-B-05 y SIS-B-06 cerrados contra f865969
SIS-B-05 y SIS-B-06 pasan de Pendiente a Cerrado. SIS-A-07 conserva su cierre
de S2 y suma el de S18, que es el de fondo: la division retirada era el sintoma
y el docstring seguia prometiendo algo que nadie comprobaba.

NOR-MEM-01, MAT-O13, NOR-HID-04 y SIS-D-05 ya estaban cerrados y se anota lo
que S18 les anadio, sin tocar el commit que los cerro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012p5FFGyBpjzMcHARygmwYd
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -4467,12 +4467,12 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S5)</t>
+          <t>Claude Code (fase1, S5) + Claude Code (fase1, S18)</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr">
         <is>
-          <t>00da460 — La frase 'el rango recorre la calidad del revestimiento' sale de la cita y pasa a declararse como INTERPRETACION DEL PROYECTISTA en `constantes_normativas.TABLA_10_INTERPRETACION_PROYECTO`, que M11 imprime separada, en su propio aviso. La `fuente` de 'v_max_concreto_eleccion', `M5.NUMERAL_V3` y la nota de la §1 del manifiesto separan ahora lo que la fuente sostiene (los dos numeros son maximos: lo dice el titulo y el rotulo 'VELOCIDAD (M/S)') de lo que pone el proyecto, y citan los dos hechos que juegan en contra de la lectura de acabados: la frase que introduce la tabla ('un rango, cuyos limites se describen a continuacion') y la fila de mamposteria con un solo valor.</t>
+          <t>00da460 — La frase 'el rango recorre la calidad del revestimiento' sale de la cita y pasa a declararse como INTERPRETACION DEL PROYECTISTA en `constantes_normativas.TABLA_10_INTERPRETACION_PROYECTO`, que M11 imprime separada, en su propio aviso. La `fuente` de 'v_max_concreto_eleccion', `M5.NUMERAL_V3` y la nota de la §1 del manifiesto separan ahora lo que la fuente sostiene (los dos numeros son maximos: lo dice el titulo y el rotulo 'VELOCIDAD (M/S)') de lo que pone el proyecto, y citan los dos hechos que juegan en contra de la lectura de acabados: la frase que introduce la tabla ('un rango, cuyos limites se describen a continuacion') y la fila de mamposteria con un solo valor. || f865969 (S18) — Reforzado en S18 con la separacion TIPOGRAFICA, que es lo que la ficha pedia y que en S5 quedo como separacion de campos. El texto sale ahora del registro (`TablaNormativa.interpretacion`, del tipo `Interpretacion`, que OBLIGA a declarar lo que juega en contra) y no de una segunda redaccion en `constantes_normativas`; se imprime en su propio bloque `class='aviso interpretacion'`, con los hechos EN CONTRA delante; y un test recorre todo lo que la memoria entrecomilla como literal y falla si la interpretacion aparece dentro de alguno.</t>
         </is>
       </c>
     </row>
@@ -4749,12 +4749,12 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S5)</t>
+          <t>Claude Code (fase1, S5) + Claude Code (fase1, S18)</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
         <is>
-          <t>00da460 — Cerrado sobre el PRODUCTO, que era donde fallaba. El matiz viajaba solo dentro de `M5.NUMERAL_V2`, o sea dentro de la tabla de verificaciones del punto, que no se imprime si el punto no llego a evaluarse -- y no llega, porque 'homogeneidad_serie_fen' bloquea el Q de la Familia A. Se agrega `constantes_normativas.UMBRALES_DE_VERIFICACION` (V1, V2, V3, TR y D_min con numeral, caracter, texto literal y lo que el proyecto hace con cada uno), `M11.bloque_umbrales()` y el marcador %%bloque_umbrales en las dos plantillas, en la seccion nueva '0-ter. Umbrales normativos y su caracter', que se imprime siempre. Medido sobre la memoria generada con tests/ejemplo_puntos.csv en los dos alcances: 'recomend' pasa de 0 a 7 apariciones y 'sedimentaci' de 0 a 3. || 76791d0 -- ademas, la memoria imprimia 'num. MC-HHD (...), num. 3.6' porque M11 anteponia 'num.' a un NUMERAL_TR que ya lo trae; y NUMERAL_V3 remitia a un simbolo de codigo que un revisor con el PDF no puede resolver.</t>
+          <t>00da460 — Cerrado sobre el PRODUCTO, que era donde fallaba. El matiz viajaba solo dentro de `M5.NUMERAL_V2`, o sea dentro de la tabla de verificaciones del punto, que no se imprime si el punto no llego a evaluarse -- y no llega, porque 'homogeneidad_serie_fen' bloquea el Q de la Familia A. Se agrega `constantes_normativas.UMBRALES_DE_VERIFICACION` (V1, V2, V3, TR y D_min con numeral, caracter, texto literal y lo que el proyecto hace con cada uno), `M11.bloque_umbrales()` y el marcador %%bloque_umbrales en las dos plantillas, en la seccion nueva '0-ter. Umbrales normativos y su caracter', que se imprime siempre. Medido sobre la memoria generada con tests/ejemplo_puntos.csv en los dos alcances: 'recomend' pasa de 0 a 7 apariciones y 'sedimentaci' de 0 a 3. || 76791d0 -- ademas, la memoria imprimia 'num. MC-HHD (...), num. 3.6' porque M11 anteponia 'num.' a un NUMERAL_TR que ya lo trae; y NUMERAL_V3 remitia a un simbolo de codigo que un revisor con el PDF no puede resolver. || f865969 (S18) — Reforzado en S18 y medido de nuevo sobre el producto. El matiz ya no viaja solo dentro del bloque fijo de umbrales: cada `PasoDeMemoria` de V2 lo lleva en su `Umbral` (caracter leido de la cita, no redactado a mano) y en `nota_del_proyecto`. Ademas se separaron las DOS MITADES del parrafo, que tienen fuerza distinta y se leian como una: 'se debera verificar' es EXIGENCIA (cita nueva `MC_HHD.4.1.1.3.6#VMIN_INICIO`, que vivia dentro de una `nota` y por eso no se podia imprimir aparte) y 'recomendandose que la velocidad minima sea igual a 0.25 m/s' es RECOMENDACION sobre el valor. Leida solo la segunda, 'V2 es una recomendacion' se entiende como que verificar el piso es opcional.</t>
         </is>
       </c>
     </row>
@@ -6579,12 +6579,12 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S5)</t>
+          <t>Claude Code (fase1, S5) + Claude Code (fase1, S18)</t>
         </is>
       </c>
       <c r="L80" s="6" t="inlineStr">
         <is>
-          <t>00da460 — `M5.NUMERAL_V1` deja de ser el numeral pelado: lleva RD, pag. impresa 79, el texto literal del 4.1.1.3.7 b) y el matiz de RECOMENDACION, igual que NUMERAL_V2, mas la declaracion de que el proyecto lo aplica como umbral duro. El comportamiento no cambia. Verificado contra el PDF: 'Se recomienda que el diseño hidraulico considere como minimo el 25 % de la altura, diametro o flecha de la estructura' (pag. impresa 79).</t>
+          <t>00da460 — `M5.NUMERAL_V1` deja de ser el numeral pelado: lleva RD, pag. impresa 79, el texto literal del 4.1.1.3.7 b) y el matiz de RECOMENDACION, igual que NUMERAL_V2, mas la declaracion de que el proyecto lo aplica como umbral duro. El comportamiento no cambia. Verificado contra el PDF: 'Se recomienda que el diseño hidraulico considere como minimo el 25 % de la altura, diametro o flecha de la estructura' (pag. impresa 79). || f865969 (S18) — Reforzado en S18: V1 emite `PasoDeMemoria` con el mismo aparato que V2 -- caracter RECOMENDACION leido de `MC_HHD.4.1.1.3.7b`, y la declaracion de que el proyecto lo aplica como umbral duro por decision conservadora propia -- y su fundamento `F5.V1` dice ademas que el 0.75 es la DERIVACION aritmetica del 25 % que el numeral escribe, no una cifra impresa.</t>
         </is>
       </c>
     </row>
@@ -8091,12 +8091,12 @@
       </c>
       <c r="K106" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S2)</t>
+          <t>Claude Code (fase1, S2) + Claude Code (fase1, S18)</t>
         </is>
       </c>
       <c r="L106" s="6" t="inlineStr">
         <is>
-          <t>3ea627c + 7266bfe</t>
+          <t>3ea627c + 7266bfe || f865969 (S18) — Confirmado vigente en S18: `angulo_aletas` lleva `reemplazado_por`, `fuente` PENDIENTE y `sin_consumidor`, y la columna 'Que lo resuelve' de M11 ya no imprime el enunciado del vacio como si fuera lo que lo resuelve.</t>
         </is>
       </c>
     </row>
@@ -12103,12 +12103,12 @@
       </c>
       <c r="K176" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S2)</t>
+          <t>Claude Code (fase1, S2) + Claude Code (fase1, S18)</t>
         </is>
       </c>
       <c r="L176" s="6" t="inlineStr">
         <is>
-          <t>3ea627c + 7266bfe</t>
+          <t>3ea627c + 7266bfe (S2) — `y/D` se retiro de M11 y vive en `ResultadoPunto.y_sobre_D`, escrito una vez. || f865969 — Cerrado DE RAIZ en S18, no solo retirando la division. M11 dejo de RECONSTRUIR la memoria: las funciones de calculo emiten `PasoDeMemoria` (§4.4) y M11 formatea. La frase del docstring 'sin calcular nada nuevo' pasa de intencion a propiedad comprobada -- `test_memoria_sustentada.test_M11_no_calcula_y_sobre_D` barre el AST del modulo y falla ante cualquier BinOp de division sobre magnitudes.</t>
         </is>
       </c>
     </row>
@@ -12596,11 +12596,19 @@
       <c r="I185" s="6" t="inlineStr"/>
       <c r="J185" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K185" s="6" t="inlineStr"/>
-      <c r="L185" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K185" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S18)</t>
+        </is>
+      </c>
+      <c r="L185" s="6" t="inlineStr">
+        <is>
+          <t>f865969 — El analisis de sensibilidad llega al documento. `_sensibilidad_declarada` imprime el rango como ANALISIS -- valor adoptado dentro de que margen, y si un barrido lo puede recorrer o no, consultando `parametros_sensibilizables(solo_numericos=True)`, que asi deja de tener por unico consumidor a los tests --. Va acompanado de la procedencia R1 de cada eleccion (`_de_donde_sale_el_valor`, que lee `Criterio.resolucion`), que era la mitad que faltaba: `_de_donde_salio` solo disparaba para lo declarado por la ventana emergente, o sea para casi nada de lo que gobierna una corrida.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="inlineStr">
@@ -12646,11 +12654,19 @@
       <c r="I186" s="6" t="inlineStr"/>
       <c r="J186" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K186" s="6" t="inlineStr"/>
-      <c r="L186" s="6" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K186" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code (fase1, S18)</t>
+        </is>
+      </c>
+      <c r="L186" s="6" t="inlineStr">
+        <is>
+          <t>f865969 — Cerrado en las dos direcciones. (1) Las dos plantillas llevan ya los MISMOS marcadores -- el contrato que el docstring de la CLI promete -- y quien decide que va dentro de `bloque_pendientes` es el ALCANCE de la corrida, que es de donde tenia que salir la decision: a nivel de perfil no se vuelca Tableros 1-2-3 y se DICE, en vez de desaparecer con el marcador. (2) `memoria_html` se detiene con ValueError si la plantilla que se le pasa no imprime un bloque que ESA corrida si produjo, medido sobre el contenido real y no sobre la lista de marcadores. El test `test_la_de_perfil_usa_un_subconjunto_estricto` EXIGIA la omision, o sea vigilaba el defecto: se reescribio como `test_las_dos_plantillas_comparten_EL_MISMO_contrato_de_marcadores` diciendo por que.</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fase1(S19b): tracker — lo que la refutacion cambio en seis fichas
Anotado contra f175fab, sin cambiar ningun Estado: los seis hallazgos cuyo
cierre la pasada adversarial obligo a precisar o a rehacer.

  SIS-A-14  el peor cerrado de la sesion: el docstring declaraba deliberado un
            comportamiento que DESTRUIA criterios_adoptados.py sin lanzar.
  SIS-A-08  el guardian que S19 escribio era vacuo en su mitad de ciclo.
  SIS-G-03  tres precisiones: las cifras eran otras, la guardia nueva se
            satisfacia sola, y una reparacion habia cambiado una referencia
            rota por otra.
  SIS-B-18  al JSON no llega: se cerraba sobre media acusacion.
  SIS-C-12  la razon escrita al cerrarlo era falsa.
  SIS-B-07  dos afirmaciones mas fuertes que el codigo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SimtPgboy5NPxdHiNTsLzK
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -12162,7 +12162,7 @@
       </c>
       <c r="L177" s="6" t="inlineStr">
         <is>
-          <t>a227cb9+e3f36df+f1b40b2+9822880 — [C11/F5, de paso] retirada del docstring de MD la premisa «M5 todavia no existe en el repositorio», que era falsa y sostenia la justificacion del Protocol y de la importacion perezosa. || S19 — REABIERTO Y VUELTO A CERRAR, porque estaba cerrado solo en su letra. La premisa falsa «M5 todavia no existe en el repositorio» se habia retirado de MD.py y sustituido por otra razon --- «la importacion perezosa evita ademas un ciclo de importacion en el arranque» --- que TAMBIEN ES FALSA: M5 importa criterios_adoptados, constantes_normativas, modelos, M2, M8 y tolerancias, y ninguno vuelve a MD. Sustituir una premisa falsa por otra no cierra el hallazgo: le cambia el hecho. Ademas la premisa original sobrevivia VERBATIM en el docstring de tests/test_MD.py, remitiendo a un parrafo de MD que ya no dice eso. Corregidas las dos, con la razon que si se sostiene, y con guardia: test_la_premisa_de_que_M5_no_existe_no_vuelve_como_afirmacion mira los docstrings POR AST y admite la mencion solo cuando el parrafo la declara caducada --- la leccion de FACTOR_MURO_TABLA.</t>
+          <t>a227cb9+e3f36df+f1b40b2+9822880 — [C11/F5, de paso] retirada del docstring de MD la premisa «M5 todavia no existe en el repositorio», que era falsa y sostenia la justificacion del Protocol y de la importacion perezosa. || S19 — REABIERTO Y VUELTO A CERRAR, porque estaba cerrado solo en su letra. La premisa falsa «M5 todavia no existe en el repositorio» se habia retirado de MD.py y sustituido por otra razon --- «la importacion perezosa evita ademas un ciclo de importacion en el arranque» --- que TAMBIEN ES FALSA: M5 importa criterios_adoptados, constantes_normativas, modelos, M2, M8 y tolerancias, y ninguno vuelve a MD. Sustituir una premisa falsa por otra no cierra el hallazgo: le cambia el hecho. Ademas la premisa original sobrevivia VERBATIM en el docstring de tests/test_MD.py, remitiendo a un parrafo de MD que ya no dice eso. Corregidas las dos, con la razon que si se sostiene, y con guardia: test_la_premisa_de_que_M5_no_existe_no_vuelve_como_afirmacion mira los docstrings POR AST y admite la mencion solo cuando el parrafo la declara caducada --- la leccion de FACTOR_MURO_TABLA. || REFUTADO EN f175fab: el guardian que S19 escribio era VACUO en su mitad de ciclo (partia nodo.module por el punto y se quedaba con 'modulos', su segunda clausula era una tautologia, y solo miraba ImportFrom). Un test verde sobre el comentario, que es el precedente FACTOR_MURO_TABLA cometido en el docstring que lo invoca para presumir de no cometerlo. Reescrito como cierre transitivo sobre Import e ImportFrom; mata el ciclo directo y el indirecto.</t>
         </is>
       </c>
     </row>
@@ -12452,7 +12452,7 @@
       </c>
       <c r="L182" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — El docstring de `escribir_valor_en_archivo` decia 'reescribe el valor=None' y el patron es `valor=)([^,\n]*)(,)`, que casa con lo que haya: un criterio YA declarado se reescribe por la misma via y el boton de la GUI esta disponible para toda fila. Es DELIBERADO --- corregir un valor adoptado es tan legitimo como declararlo, y obligar a editar el archivo a mano empujaria a saltarse la guardia --- y lo que faltaba era decirlo. Queda escrito ademas lo que la funcion NO toca (etiqueta, justificacion, fuente, sensibilidad, resolucion) y que la GUI lo advierte en su confirmacion.</t>
+          <t>4141fd5 — El docstring de `escribir_valor_en_archivo` decia 'reescribe el valor=None' y el patron es `valor=)([^,\n]*)(,)`, que casa con lo que haya: un criterio YA declarado se reescribe por la misma via y el boton de la GUI esta disponible para toda fila. Es DELIBERADO --- corregir un valor adoptado es tan legitimo como declararlo, y obligar a editar el archivo a mano empujaria a saltarse la guardia --- y lo que faltaba era decirlo. Queda escrito ademas lo que la funcion NO toca (etiqueta, justificacion, fuente, sensibilidad, resolucion) y que la GUI lo advierte en su confirmacion. || REFUTADO Y REABIERTO EN f175fab, y era lo peor cerrado de la sesion. El docstring declaraba «REESCRIBE CUALQUIER VALOR ... es deliberado» y para cuatro criterios --- F_pga, hds5_embocadura_hdpe, diametros_normalizados, D_max_catalogo --- no reescribia: DESTRUIA criterios_adoptados.py dejandolo con SyntaxError y VOLVIA SIN EXCEPCION. El patron se corta en la primera coma y un valor de UNA LINEA con comas quedaba partido. La GUI pintaba «escrito» en verde y, como refresca CRITERIOS en memoria, la corrupcion no aparecia hasta el siguiente arranque. Es el mismo desastre que SIS-F-19 describe para los MULTILINEA, en el hueco que ese test no cubria. Guardia: ast.parse sobre el texto resultante ANTES de escribir, mas dos tests. Y el Tooltip del boton --- lo que lee el USUARIO --- seguia diciendo «Reescribe 'valor=None'»: la correccion habia llegado solo a quien lee el codigo.</t>
         </is>
       </c>
     </row>
@@ -13783,7 +13783,7 @@
       </c>
       <c r="L205" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — CONSERVADO con su razon escrita, y la razon es mas fuerte que 'la otra via es mas rica': la via del `Bloqueo` es la UNICA. Comprobado vaciando el valor de los 46 criterios y de todos los datos de sitio: cli.correr devuelve informe sin levantar nada, con 12 bloqueos archivados. Los tres unicos sitios que levantan CriterioPendienteError cuelgan de etapas envueltas por _etapa, de modo que ninguno alcanza el except ErrorProyecto de la ventana. El docstring afirmaba un estado falso ('Texto que la GUI muestra al usuario') y se reescribio. DEFECTO CONTRA CLAUDE.md CORREGIDO: su clausula decia que la GUI muestra 'falta declarar: &lt;clave&gt;' y la GUI pinta seis columnas por `M11.criterios_bloqueantes`. Ficha en docs/decisiones_diferidas.md.</t>
+          <t>4141fd5 — CONSERVADO con su razon escrita, y la razon es mas fuerte que 'la otra via es mas rica': la via del `Bloqueo` es la UNICA. Comprobado vaciando el valor de los 46 criterios y de todos los datos de sitio: cli.correr devuelve informe sin levantar nada, con 12 bloqueos archivados. Los tres unicos sitios que levantan CriterioPendienteError cuelgan de etapas envueltas por _etapa, de modo que ninguno alcanza el except ErrorProyecto de la ventana. El docstring afirmaba un estado falso ('Texto que la GUI muestra al usuario') y se reescribio. DEFECTO CONTRA CLAUDE.md CORREGIDO: su clausula decia que la GUI muestra 'falta declarar: &lt;clave&gt;' y la GUI pinta seis columnas por `M11.criterios_bloqueantes`. Ficha en docs/decisiones_diferidas.md. || PRECISADO EN f175fab: «[N] imposible» y el censo de lo que corre fuera de `_etapa` eran afirmaciones mas fuertes que el codigo. Sustituidas por lo comprobable.</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="L215" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — La ficha esta obsoleta en LA MITAD de su acusacion --- «no se emite ni al JSON ni al HTML» --- y la otra mitad sigue viva. Al HTML SI llega: `ahogado_por_TW` SI tiene lector de produccion y SI llega a la memoria desde S18 (f865969), dentro del PasoDeMemoria de h_o que emite `M4._pasos_hidraulicos` --- «(manda TW: la salida esta ahogada)» frente a «(manda la aproximacion geometrica)» ---. Se cerro solo, sin que nadie marcara el hallazgo. S19 lo verifica ejecutando las dos ramas, lo escribe en el docstring de `ControlSalida` y lo FIJA con un test sobre el TEXTO RENDERIZADO, no sobre el booleano: hasta ahora el campo asomaba al entregable por una sola frase y nada la protegia. AL JSON NO LLEGA, y eso no se cierra aqui: no llega ninguna pieza del bloque h_o (`grep -n 'h_o' cli.py` esta vacio), ni siquiera los dos flags de condicion de uso. Publicar la etiqueta de la rama sin h_o, TW ni la aproximacion geometrica daria al lector del JSON un veredicto sin los dos numeros que lo producen, que es menos revisable que no publicar nada. Abrir el JSON al bloque h_o ENTERO es una decision propia y no parte de SIS-B-18. Los otros cuatro campos siguen con su decision escrita, como la ficha reconoce. HALLAZGO NUEVO ABIERTO DE PASO: `M9_cabezal.combinaciones()` afirmaba en su docstring que 'M11 la usa' y M11 no la referencia --- corregido, con la razon de por que se conserva.</t>
+          <t>4141fd5 — La ficha esta obsoleta en LA MITAD de su acusacion --- «no se emite ni al JSON ni al HTML» --- y la otra mitad sigue viva. Al HTML SI llega: `ahogado_por_TW` SI tiene lector de produccion y SI llega a la memoria desde S18 (f865969), dentro del PasoDeMemoria de h_o que emite `M4._pasos_hidraulicos` --- «(manda TW: la salida esta ahogada)» frente a «(manda la aproximacion geometrica)» ---. Se cerro solo, sin que nadie marcara el hallazgo. S19 lo verifica ejecutando las dos ramas, lo escribe en el docstring de `ControlSalida` y lo FIJA con un test sobre el TEXTO RENDERIZADO, no sobre el booleano: hasta ahora el campo asomaba al entregable por una sola frase y nada la protegia. AL JSON NO LLEGA, y eso no se cierra aqui: no llega ninguna pieza del bloque h_o (`grep -n 'h_o' cli.py` esta vacio), ni siquiera los dos flags de condicion de uso. Publicar la etiqueta de la rama sin h_o, TW ni la aproximacion geometrica daria al lector del JSON un veredicto sin los dos numeros que lo producen, que es menos revisable que no publicar nada. Abrir el JSON al bloque h_o ENTERO es una decision propia y no parte de SIS-B-18. Los otros cuatro campos siguen con su decision escrita, como la ficha reconoce. HALLAZGO NUEVO ABIERTO DE PASO: `M9_cabezal.combinaciones()` afirmaba en su docstring que 'M11 la usa' y M11 no la referencia --- corregido, con la razon de por que se conserva. || PRECISADO EN f175fab: al JSON NO llega, y el cierre anterior daba la ficha por obsoleta entera. Se declara que abrir el JSON al bloque h_o completo es decision propia.</t>
         </is>
       </c>
     </row>
@@ -14598,7 +14598,7 @@
       </c>
       <c r="L219" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — Y EL HALLAZGO SE QUEDABA CORTO, dicho para que no se lea de menos: no era solo que el ejemplo diera las luces sin la salvedad que si lleva el test y con ids del fixture presentados como cruces reales --- es que NO EJECUTABA. Llamaba a `clasificar_puntos` con dos de sus tres argumentos y abortaba en el primer punto con CriterioPendienteError sobre 'umbral_area_quebrada_importante_ha' (reproducido). El bloque Uso nuevo corre y da 71/35/35/None, dice que los ids son del fixture y que la luz no es columna de la Sec. 1.2, y corrige '# detiene los puentes', que describia un efecto que con esas cuatro luces no se produce. Lo fija un test que EXTRAE el bloque del archivo y lo ejecuta, de modo que ejemplo y test no puedan volver a divergir.</t>
+          <t>4141fd5 — Y EL HALLAZGO SE QUEDABA CORTO, dicho para que no se lea de menos: no era solo que el ejemplo diera las luces sin la salvedad que si lleva el test y con ids del fixture presentados como cruces reales --- es que NO EJECUTABA. Llamaba a `clasificar_puntos` con dos de sus tres argumentos y abortaba en el primer punto con CriterioPendienteError sobre 'umbral_area_quebrada_importante_ha' (reproducido). El bloque Uso nuevo corre y da 71/35/35/None, dice que los ids son del fixture y que la luz no es columna de la Sec. 1.2, y corrige '# detiene los puentes', que describia un efecto que con esas cuatro luces no se produce. Lo fija un test que EXTRAE el bloque del archivo y lo ejecuta, de modo que ejemplo y test no puedan volver a divergir. || PRECISADO EN f175fab: la razon escrita al cerrarlo --- «los otros doce bloques Uso son fragmentos a proposito» --- era FALSA; los de M0_carga y M10_espaciamiento corren enteros. Es el mismo defecto que la ficha denuncia, cometido al cerrarla. Hoy la suite EJECUTA los tres que se sostienen solos y un segundo test hace crecer la lista si alguien arregla otro.</t>
         </is>
       </c>
     </row>
@@ -15631,7 +15631,7 @@
       </c>
       <c r="L238" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — EL BARRIDO QUE LA FICHA PEDIA, HECHO, y el hueco del test cerrado por cambio de diseño. La ficha decia que la tasa entre las no ancladas era DESCONOCIDA: medida, era mala. De 68 referencias no ancladas, 16 llevaban a un sitio que no habla de lo que la fila dice --- entre ellas `e2_volteo()` y `empuje_flotacion()`, nombres que el codigo ya no tiene, y ESPACIAMIENTO_MAX_VECES_ESPESOR apuntando al bloque de `n_s_zapata_en_talud` --- y de las 32 restantes sin identificador, 27 tambien. Todas verificadas LEYENDO la linea de destino y reparadas. EL CAMBIO DE DISEÑO: «de prosa» mezclaba dos poblaciones, la fila que no nombra nada (hueco real) y la que nombra un simbolo que el archivo USA sin definir (verificable). Separadas: `test_toda_fila_que_cita_un_identificador_lo_nombra_en_su_destino`, SIN CUPO. Ademas: `_simbolos_citados` devuelve la cola punteada (`M9.cuantia_de_diseno`) y filtra ids de ficha --- eso solo destapo 4 desviadas ---; el resincronizador aprende a mantener las referencias por mencion; y se retiran 40 etiquetas con rango IMPOSIBLE (`[CN:170-49]`), defecto nunca reportado que nacia de reescribir el inicio conservando el final viejo. RESULTADO: 326 referencias = 299 por simbolo + 25 por mencion + 2 sin identificador (las dos legitimas, a docstring de modulo), 0 rotas. Cupos bajados 82-&gt;27 y 33-&gt;2, cobertura verificable del 99 %.</t>
+          <t>4141fd5 — EL BARRIDO QUE LA FICHA PEDIA, HECHO, y el hueco del test cerrado por cambio de diseño. La ficha decia que la tasa entre las no ancladas era DESCONOCIDA: medida, era mala. De 68 referencias no ancladas, 16 llevaban a un sitio que no habla de lo que la fila dice --- entre ellas `e2_volteo()` y `empuje_flotacion()`, nombres que el codigo ya no tiene, y ESPACIAMIENTO_MAX_VECES_ESPESOR apuntando al bloque de `n_s_zapata_en_talud` --- y de las 32 restantes sin identificador, 27 tambien. Todas verificadas LEYENDO la linea de destino y reparadas. EL CAMBIO DE DISEÑO: «de prosa» mezclaba dos poblaciones, la fila que no nombra nada (hueco real) y la que nombra un simbolo que el archivo USA sin definir (verificable). Separadas: `test_toda_fila_que_cita_un_identificador_lo_nombra_en_su_destino`, SIN CUPO. Ademas: `_simbolos_citados` devuelve la cola punteada (`M9.cuantia_de_diseno`) y filtra ids de ficha --- eso solo destapo 4 desviadas ---; el resincronizador aprende a mantener las referencias por mencion; y se retiran 40 etiquetas con rango IMPOSIBLE (`[CN:170-49]`), defecto nunca reportado que nacia de reescribir el inicio conservando el final viejo. RESULTADO: 326 referencias = 299 por simbolo + 25 por mencion + 2 sin identificador (las dos legitimas, a docstring de modulo), 0 rotas. Cupos bajados 82-&gt;27 y 33-&gt;2, cobertura verificable del 99 %. || PRECISADO EN f175fab tras la refutacion, en tres cosas. (1) LAS CIFRAS ERAN OTRAS: medido con la regla final sobre f56360c, eran 20 rotas de 64 no ancladas (no 16 de 68) y 50 etiquetas con rango imposible (no 40 ni 48). (2) LA GUARDIA NUEVA SE SATISFACIA SOLA: comprobaba el BLOQUE, y seis referencias saboteadas --- una a OTRO ARCHIVO, otra a 2900 lineas de su uso --- pasaban con la suite en verde. Ahora comprueba EL PARRAFO DE LLEGADA y el resincronizador ancla al RENGLON, no al bloque; ademas se descartan los tokens que no son simbolos del proyecto (`py`, cola de un backtick `constantes_normativas.py`, hacia de comodin). (3) UNA REPARACION HABIA CAMBIADO UNA REFERENCIA ROTA POR OTRA: la fila de GAMMA_AGUA_KN_M3 aterrizaba en G_LAUSHEY_ATRIBUCION y la salvaba un comentario que dice que el simbolo NO esta ahi. Reapuntada a constantes_fisicas.py, y la fila corregida ademas de fondo: dejo de ser [N].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fase1(S19c): tracker — SIS-F-13 y SIS-A-01 anotados contra 4047fb6
Ningun Estado cambia. Se anota lo que la refutacion de los tests nuevos
obligo a rehacer: la guardia de SIS-F-13 decidia por subcadena (cometia
SIS-F-17 al cerrarlo) y la de SIS-A-01 era verde sobre la mencion del simbolo,
de modo que el hallazgo bloqueante del expediente se podia reabrir con la
suite entera en verde.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SimtPgboy5NPxdHiNTsLzK
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -2032,7 +2032,7 @@
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>3ea627c + 7266bfe</t>
+          <t>3ea627c + 7266bfe || S19c: la guardia que S19 le puso en la GUI era VERDE SOBRE LA MENCION del simbolo. `test_la_tabla_de_criterios_muestra_el_valor_efectivo_y_no_lo_recalcula` solo comprobaba que `ca.criterio_efectivo` apareciera como llamada en el AST, de modo que el hallazgo se reabria dejando la llamada en su sitio y leyendo el valor del ARCHIVO: la fila quedaba rotulada «declarado (corrida)» y con «(sin declarar)» en su columna de valor --- contradiciendose en pantalla --- y la suite entera en verde. Ahora se sigue el DATO: que nombre recibe `criterio_efectivo(...).valor` y que ese nombre entre en el `values=` del `insert`. El estado no cambia (sigue Cerrado desde S2); lo que cambia es que ahora esta defendido.</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="L140" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — RAZON ESTRECHADA DE TRES A DOS. `test_M5_verificaciones.py` consume ya CP-3 por la cadena de produccion entera (catalogo de M2 -&gt; Manning de M3 -&gt; umbral de M5) sin fabricar ningun dorado: todos los numeros salen de CP-2, CP-3 o de la constante [N] V_MIN, de modo que el conflicto n.7 no se toca. CP-3 gana ademas su propia `tolerancia_V` declarada, y test_M3 deja de escribirla a mano. Y LA REGLA DEJA DE VIVIR SOLO EN CLAUDE.md: test_guardias_de_la_suite.test_todo_modulo_de_calculo_consume_su_caso_patron la ejecuta, con la lista de exentos DECLARADA (M2, M8, M10 con la fuente que falta segun la §15; M11 por no corresponderle dorado) y fallando tambien si un exento deja de serlo. SIGUEN SIN CASO PATRON M2, M8 y M10, por falta de fuente externa: A796/A796M no esta en normas/, y para M10 lo que falta no es una norma sino el expediente vial.</t>
+          <t>4141fd5 — RAZON ESTRECHADA DE TRES A DOS. `test_M5_verificaciones.py` consume ya CP-3 por la cadena de produccion entera (catalogo de M2 -&gt; Manning de M3 -&gt; umbral de M5) sin fabricar ningun dorado: todos los numeros salen de CP-2, CP-3 o de la constante [N] V_MIN, de modo que el conflicto n.7 no se toca. CP-3 gana ademas su propia `tolerancia_V` declarada, y test_M3 deja de escribirla a mano. Y LA REGLA DEJA DE VIVIR SOLO EN CLAUDE.md: test_guardias_de_la_suite.test_todo_modulo_de_calculo_consume_su_caso_patron la ejecuta, con la lista de exentos DECLARADA (M2, M8, M10 con la fuente que falta segun la §15; M11 por no corresponderle dorado) y fallando tambien si un exento deja de serlo. SIGUEN SIN CASO PATRON M2, M8 y M10, por falta de fuente externa: A796/A796M no esta en normas/, y para M10 lo que falta no es una norma sino el expediente vial. || PRECISADO EN S19c tras refutar los tests nuevos: la guardia que se escribio para cerrar este hallazgo decidia si un modulo consume su caso patron con `"casos_patron" in texto`, una busqueda de subcadena --- o sea que cometia SIS-F-17 al cerrar SIS-F-13 ---. Fallaba en las dos direcciones: un modulo podia perder el import Y el test y quedar verde mientras sobreviviera la palabra en un comentario, y un exento que solo la mencionara disparaba la alarma contraria. Reescrita por AST; el mutante muere. Y los DOS tests de CP-3 se rehicieron: el primero anunciaba vigilar la tolerancia de umbral y no la vigila (margen 7.3e-06 contra TOL 1e-09), y el segundo decia ejercitar la conclusion del fixture evaluando FUERA de sus condiciones (y/D caia a 0.32 desde el 0.75 que la conclusion fija). El segundo se reescribio sobre la mitad que nadie ejercitaba: la salvedad de MAT-O20 --- «con y/D &lt; 0.056 V2 SI se viola a S = 0.001» --- era una afirmacion escrita y no comprobada, y ahora se comprueba con su frontera por los dos lados.</t>
         </is>
       </c>
     </row>

</xml_diff>